<commit_message>
fix: Tasks 'Done' date column name to match Notion DB
</commit_message>
<xml_diff>
--- a/notion-import-templates/Insurance_Policies_Template.xlsx
+++ b/notion-import-templates/Insurance_Policies_Template.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30126"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_4902661BDEE849986904A2AD6474A91100A393FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCB74C1D-C753-420D-99F3-C4E96B9D6774}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="11_4902661BDEE849986904A2AD6474A91100A393FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFB25BB2-E697-4CD8-9683-25D7C5244FDD}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12,12 +12,28 @@
     <sheet name="Reference" sheetId="2" r:id="rId2"/>
     <sheet name="Sample" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="143">
   <si>
     <t>Bill Morrisons — Insurance Policies Data Entry</t>
   </si>
@@ -303,6 +319,15 @@
   </si>
   <si>
     <t>🛡️ Life Cover, ♿ TPD, 🏥 Medical, ⏸️ Waiver of Premium</t>
+  </si>
+  <si>
+    <t>0104649955</t>
+  </si>
+  <si>
+    <t>13/06/2011</t>
+  </si>
+  <si>
+    <t>13/06/2085</t>
   </si>
   <si>
     <t>Insurance Type</t>
@@ -444,7 +469,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -473,13 +501,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
+      <alignment horizontal="center"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -490,6 +536,18 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{69E5B004-7BF1-42CC-BE29-6E2C6D39DB56}" name="Table1" displayName="Table1" ref="N3:P33" totalsRowShown="0">
+  <autoFilter ref="N3:P33" xr:uid="{69E5B004-7BF1-42CC-BE29-6E2C6D39DB56}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{58D46586-83F1-4520-BB84-8DECA7EF760D}" name="Annual Premium (MYR)"/>
+    <tableColumn id="2" xr3:uid="{0829D2FE-2862-4852-907C-03838995F0B3}" name="Commencement Date" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{8694827B-7786-4F19-9FDD-25C3897B6953}" name="Maturity Date" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -814,13 +872,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T33"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.5"/>
+  <dimension ref="A1:T34"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="7" max="7" width="12.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="106.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="68" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.75" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="35.75" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="28.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:20" ht="15.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -839,7 +906,7 @@
       <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
@@ -863,10 +930,10 @@
       <c r="N1" t="s">
         <v>1</v>
       </c>
-      <c r="O1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P1" t="s">
+      <c r="O1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Q1" t="s">
@@ -882,7 +949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:20" ht="15.75">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -901,7 +968,7 @@
       <c r="F2" t="s">
         <v>1</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H2" t="s">
@@ -925,10 +992,10 @@
       <c r="N2" t="s">
         <v>1</v>
       </c>
-      <c r="O2" t="s">
-        <v>1</v>
-      </c>
-      <c r="P2" t="s">
+      <c r="O2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Q2" t="s">
@@ -944,7 +1011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:20" ht="15.75">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -963,7 +1030,7 @@
       <c r="F3" t="s">
         <v>8</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H3" t="s">
@@ -987,10 +1054,10 @@
       <c r="N3" t="s">
         <v>16</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="1" t="s">
         <v>18</v>
       </c>
       <c r="Q3" t="s">
@@ -1006,7 +1073,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:20" ht="15.75">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -1025,7 +1092,7 @@
       <c r="F4" t="s">
         <v>28</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H4" t="s">
@@ -1049,10 +1116,10 @@
       <c r="N4" t="s">
         <v>36</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" s="1" t="s">
         <v>38</v>
       </c>
       <c r="Q4" t="s">
@@ -1068,7 +1135,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:20" ht="15.75">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1087,7 +1154,7 @@
       <c r="F5" t="s">
         <v>48</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="1" t="s">
         <v>49</v>
       </c>
       <c r="H5">
@@ -1111,10 +1178,10 @@
       <c r="N5">
         <v>5340</v>
       </c>
-      <c r="O5">
+      <c r="O5" s="3">
         <v>43444</v>
       </c>
-      <c r="P5">
+      <c r="P5" s="3">
         <v>68281</v>
       </c>
       <c r="Q5" t="s">
@@ -1130,7 +1197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:20" ht="15.75">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1149,7 +1216,7 @@
       <c r="F6" t="s">
         <v>53</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="1">
         <v>6000739155</v>
       </c>
       <c r="H6">
@@ -1173,10 +1240,10 @@
       <c r="N6">
         <v>3204</v>
       </c>
-      <c r="O6">
+      <c r="O6" s="3">
         <v>41968</v>
       </c>
-      <c r="P6">
+      <c r="P6" s="3">
         <v>68266</v>
       </c>
       <c r="Q6" t="s">
@@ -1192,7 +1259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:20" ht="15.75">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -1211,7 +1278,7 @@
       <c r="F7" t="s">
         <v>53</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="1" t="s">
         <v>56</v>
       </c>
       <c r="H7">
@@ -1235,10 +1302,10 @@
       <c r="N7">
         <v>1200</v>
       </c>
-      <c r="O7">
+      <c r="O7" s="3">
         <v>41291</v>
       </c>
-      <c r="P7">
+      <c r="P7" s="3">
         <v>68319</v>
       </c>
       <c r="Q7" t="s">
@@ -1254,7 +1321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:20" ht="15.75">
       <c r="A8" t="s">
         <v>57</v>
       </c>
@@ -1273,7 +1340,7 @@
       <c r="F8" t="s">
         <v>53</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="1" t="s">
         <v>59</v>
       </c>
       <c r="H8">
@@ -1297,10 +1364,10 @@
       <c r="N8">
         <v>3960</v>
       </c>
-      <c r="O8">
+      <c r="O8" s="3">
         <v>43517</v>
       </c>
-      <c r="P8">
+      <c r="P8" s="3">
         <v>60684</v>
       </c>
       <c r="Q8" t="s">
@@ -1316,7 +1383,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:20" ht="15.75">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -1335,7 +1402,7 @@
       <c r="F9" t="s">
         <v>53</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="1" t="s">
         <v>63</v>
       </c>
       <c r="H9">
@@ -1359,10 +1426,10 @@
       <c r="N9">
         <v>1800</v>
       </c>
-      <c r="O9">
+      <c r="O9" s="3">
         <v>42252</v>
       </c>
-      <c r="P9">
+      <c r="P9" s="3">
         <v>65263</v>
       </c>
       <c r="Q9" t="s">
@@ -1378,7 +1445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:20" ht="15.75">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -1397,7 +1464,7 @@
       <c r="F10" t="s">
         <v>53</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="1">
         <v>8009558744</v>
       </c>
       <c r="H10">
@@ -1421,10 +1488,10 @@
       <c r="N10">
         <v>4020</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="3">
         <v>45783</v>
       </c>
-      <c r="P10">
+      <c r="P10" s="3">
         <v>54184</v>
       </c>
       <c r="Q10" t="s">
@@ -1440,7 +1507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:20" ht="15.75">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1459,7 +1526,7 @@
       <c r="F11" t="s">
         <v>53</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="1">
         <v>8001890884</v>
       </c>
       <c r="H11">
@@ -1483,10 +1550,10 @@
       <c r="N11">
         <v>1800</v>
       </c>
-      <c r="O11">
+      <c r="O11" s="3">
         <v>43309</v>
       </c>
-      <c r="P11">
+      <c r="P11" s="3">
         <v>79103</v>
       </c>
       <c r="Q11" t="s">
@@ -1502,7 +1569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:20" ht="15.75">
       <c r="A12" t="s">
         <v>66</v>
       </c>
@@ -1521,7 +1588,7 @@
       <c r="F12" t="s">
         <v>53</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="1">
         <v>8010673726</v>
       </c>
       <c r="H12">
@@ -1545,10 +1612,10 @@
       <c r="N12">
         <v>1896</v>
       </c>
-      <c r="O12">
+      <c r="O12" s="3">
         <v>46092</v>
       </c>
-      <c r="P12">
+      <c r="P12" s="3">
         <v>71660</v>
       </c>
       <c r="Q12" t="s">
@@ -1564,7 +1631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:20" ht="15.75">
       <c r="A13" t="s">
         <v>66</v>
       </c>
@@ -1583,7 +1650,7 @@
       <c r="F13" t="s">
         <v>53</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="1">
         <v>8010673637</v>
       </c>
       <c r="H13">
@@ -1607,10 +1674,10 @@
       <c r="N13">
         <v>5604</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="3">
         <v>46092</v>
       </c>
-      <c r="P13">
+      <c r="P13" s="3">
         <v>57415</v>
       </c>
       <c r="Q13" t="s">
@@ -1626,7 +1693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:20" ht="15.75">
       <c r="A14" t="s">
         <v>66</v>
       </c>
@@ -1645,7 +1712,7 @@
       <c r="F14" t="s">
         <v>53</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="1">
         <v>6001000871</v>
       </c>
       <c r="H14">
@@ -1669,10 +1736,10 @@
       <c r="N14">
         <v>2400</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="3">
         <v>42142</v>
       </c>
-      <c r="P14">
+      <c r="P14" s="3">
         <v>64788</v>
       </c>
       <c r="Q14" t="s">
@@ -1688,7 +1755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:20" ht="15.75">
       <c r="A15" t="s">
         <v>66</v>
       </c>
@@ -1707,7 +1774,7 @@
       <c r="F15" t="s">
         <v>72</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="1">
         <v>35438762</v>
       </c>
       <c r="H15">
@@ -1731,10 +1798,10 @@
       <c r="N15">
         <v>7392</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="3">
         <v>43344</v>
       </c>
-      <c r="P15">
+      <c r="P15" s="3">
         <v>64529</v>
       </c>
       <c r="Q15" t="s">
@@ -1750,7 +1817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:20" ht="15.75">
       <c r="A16" t="s">
         <v>66</v>
       </c>
@@ -1769,7 +1836,7 @@
       <c r="F16" t="s">
         <v>72</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="1">
         <v>31359163</v>
       </c>
       <c r="H16">
@@ -1793,10 +1860,10 @@
       <c r="N16">
         <v>5868.6</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="3">
         <v>45292</v>
       </c>
-      <c r="P16">
+      <c r="P16" s="3">
         <v>57346</v>
       </c>
       <c r="Q16" t="s">
@@ -1812,7 +1879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:20" ht="15.75">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -1831,7 +1898,7 @@
       <c r="F17" t="s">
         <v>72</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="1">
         <v>35439348</v>
       </c>
       <c r="H17">
@@ -1855,10 +1922,10 @@
       <c r="N17">
         <v>6924</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="3">
         <v>43344</v>
       </c>
-      <c r="P17">
+      <c r="P17" s="3">
         <v>66355</v>
       </c>
       <c r="Q17" t="s">
@@ -1874,7 +1941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:20" ht="15.75">
       <c r="A18" t="s">
         <v>68</v>
       </c>
@@ -1893,7 +1960,7 @@
       <c r="F18" t="s">
         <v>53</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="1">
         <v>6000739226</v>
       </c>
       <c r="H18">
@@ -1917,10 +1984,10 @@
       <c r="N18">
         <v>2400</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="3">
         <v>41969</v>
       </c>
-      <c r="P18">
+      <c r="P18" s="3">
         <v>66806</v>
       </c>
       <c r="Q18" t="s">
@@ -1936,7 +2003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:20" ht="15.75">
       <c r="A19" t="s">
         <v>68</v>
       </c>
@@ -1955,7 +2022,7 @@
       <c r="F19" t="s">
         <v>53</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="1">
         <v>8010673612</v>
       </c>
       <c r="H19">
@@ -1979,10 +2046,10 @@
       <c r="N19">
         <v>4200</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="3">
         <v>46092</v>
       </c>
-      <c r="P19">
+      <c r="P19" s="3">
         <v>59241</v>
       </c>
       <c r="Q19" t="s">
@@ -1998,7 +2065,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:20" ht="15.75">
       <c r="A20" t="s">
         <v>77</v>
       </c>
@@ -2017,7 +2084,7 @@
       <c r="F20" t="s">
         <v>53</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="1">
         <v>8010751037</v>
       </c>
       <c r="H20">
@@ -2041,10 +2108,10 @@
       <c r="N20">
         <v>1824</v>
       </c>
-      <c r="O20">
+      <c r="O20" s="3">
         <v>46111</v>
       </c>
-      <c r="P20">
+      <c r="P20" s="3">
         <v>69850</v>
       </c>
       <c r="Q20" t="s">
@@ -2060,7 +2127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:20" ht="15.75">
       <c r="A21" t="s">
         <v>77</v>
       </c>
@@ -2079,7 +2146,7 @@
       <c r="F21" t="s">
         <v>53</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="1">
         <v>8010750874</v>
       </c>
       <c r="H21">
@@ -2103,10 +2170,10 @@
       <c r="N21">
         <v>4248</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="3">
         <v>46111</v>
       </c>
-      <c r="P21">
+      <c r="P21" s="3">
         <v>60719</v>
       </c>
       <c r="Q21" t="s">
@@ -2122,7 +2189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:20" ht="15.75">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -2141,7 +2208,7 @@
       <c r="F22" t="s">
         <v>53</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="1">
         <v>8010750804</v>
       </c>
       <c r="H22">
@@ -2165,10 +2232,10 @@
       <c r="N22">
         <v>1848</v>
       </c>
-      <c r="O22">
+      <c r="O22" s="3">
         <v>46111</v>
       </c>
-      <c r="P22">
+      <c r="P22" s="3">
         <v>68389</v>
       </c>
       <c r="Q22" t="s">
@@ -2184,7 +2251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:20" ht="15.75">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -2203,7 +2270,7 @@
       <c r="F23" t="s">
         <v>53</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="1">
         <v>8003557527</v>
       </c>
       <c r="H23">
@@ -2227,10 +2294,10 @@
       <c r="N23">
         <v>1800</v>
       </c>
-      <c r="O23">
+      <c r="O23" s="3">
         <v>43859</v>
       </c>
-      <c r="P23">
+      <c r="P23" s="3">
         <v>54816</v>
       </c>
       <c r="Q23" t="s">
@@ -2246,7 +2313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:20" ht="15.75">
       <c r="A24" t="s">
         <v>77</v>
       </c>
@@ -2265,7 +2332,7 @@
       <c r="F24" t="s">
         <v>53</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="1">
         <v>6001564581</v>
       </c>
       <c r="H24">
@@ -2289,10 +2356,10 @@
       <c r="N24">
         <v>1800</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="3">
         <v>42621</v>
       </c>
-      <c r="P24">
+      <c r="P24" s="3">
         <v>68188</v>
       </c>
       <c r="Q24" t="s">
@@ -2308,7 +2375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:20" ht="15.75">
       <c r="A25" t="s">
         <v>77</v>
       </c>
@@ -2327,7 +2394,7 @@
       <c r="F25" t="s">
         <v>53</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="1">
         <v>8003219923</v>
       </c>
       <c r="H25">
@@ -2351,10 +2418,10 @@
       <c r="N25">
         <v>2232</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="3">
         <v>43752</v>
       </c>
-      <c r="P25">
+      <c r="P25" s="3">
         <v>51423</v>
       </c>
       <c r="Q25" t="s">
@@ -2370,7 +2437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:20" ht="15.75">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -2389,7 +2456,7 @@
       <c r="F26" t="s">
         <v>53</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="1">
         <v>8001036225</v>
       </c>
       <c r="H26">
@@ -2413,10 +2480,10 @@
       <c r="N26">
         <v>1200</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="3">
         <v>42993</v>
       </c>
-      <c r="P26">
+      <c r="P26" s="3">
         <v>79152</v>
       </c>
       <c r="Q26" t="s">
@@ -2432,7 +2499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:20" ht="15.75">
       <c r="A27" t="s">
         <v>77</v>
       </c>
@@ -2451,7 +2518,7 @@
       <c r="F27" t="s">
         <v>53</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="1">
         <v>8005353726</v>
       </c>
       <c r="H27">
@@ -2475,10 +2542,10 @@
       <c r="N27">
         <v>1200</v>
       </c>
-      <c r="O27">
+      <c r="O27" s="3">
         <v>44447</v>
       </c>
-      <c r="P27">
+      <c r="P27" s="3">
         <v>75857</v>
       </c>
       <c r="Q27" t="s">
@@ -2494,7 +2561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:20" ht="15.75">
       <c r="A28" t="s">
         <v>82</v>
       </c>
@@ -2513,7 +2580,7 @@
       <c r="F28" t="s">
         <v>53</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G28" s="1" t="s">
         <v>83</v>
       </c>
       <c r="H28">
@@ -2537,10 +2604,10 @@
       <c r="N28">
         <v>2304</v>
       </c>
-      <c r="O28">
+      <c r="O28" s="3">
         <v>41269</v>
       </c>
-      <c r="P28">
+      <c r="P28" s="3">
         <v>67932</v>
       </c>
       <c r="Q28" t="s">
@@ -2556,7 +2623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:20" ht="15.75">
       <c r="A29" t="s">
         <v>84</v>
       </c>
@@ -2575,7 +2642,7 @@
       <c r="F29" t="s">
         <v>53</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G29" s="1" t="s">
         <v>85</v>
       </c>
       <c r="H29">
@@ -2599,10 +2666,10 @@
       <c r="N29">
         <v>3744</v>
       </c>
-      <c r="O29">
+      <c r="O29" s="3">
         <v>40704</v>
       </c>
-      <c r="P29">
+      <c r="P29" s="3">
         <v>68098</v>
       </c>
       <c r="Q29" t="s">
@@ -2618,7 +2685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:20" ht="15.75">
       <c r="A30" t="s">
         <v>84</v>
       </c>
@@ -2637,7 +2704,7 @@
       <c r="F30" t="s">
         <v>53</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="1" t="s">
         <v>87</v>
       </c>
       <c r="H30">
@@ -2661,10 +2728,10 @@
       <c r="N30">
         <v>2400</v>
       </c>
-      <c r="O30">
+      <c r="O30" s="3">
         <v>41479</v>
       </c>
-      <c r="P30">
+      <c r="P30" s="3">
         <v>68142</v>
       </c>
       <c r="Q30" t="s">
@@ -2680,7 +2747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:20" ht="15.75">
       <c r="A31" t="s">
         <v>88</v>
       </c>
@@ -2699,7 +2766,7 @@
       <c r="F31" t="s">
         <v>53</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="1" t="s">
         <v>90</v>
       </c>
       <c r="H31">
@@ -2723,10 +2790,10 @@
       <c r="N31">
         <v>1200</v>
       </c>
-      <c r="O31">
+      <c r="O31" s="3">
         <v>40145</v>
       </c>
-      <c r="P31">
+      <c r="P31" s="3">
         <v>67173</v>
       </c>
       <c r="Q31" t="s">
@@ -2742,7 +2809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:20" ht="15.75">
       <c r="A32" t="s">
         <v>88</v>
       </c>
@@ -2761,7 +2828,7 @@
       <c r="F32" t="s">
         <v>53</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" s="1" t="s">
         <v>93</v>
       </c>
       <c r="H32">
@@ -2785,10 +2852,10 @@
       <c r="N32">
         <v>1200</v>
       </c>
-      <c r="O32">
+      <c r="O32" s="3">
         <v>41535</v>
       </c>
-      <c r="P32">
+      <c r="P32" s="3">
         <v>67102</v>
       </c>
       <c r="Q32" t="s">
@@ -2804,7 +2871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:20" ht="15.75">
       <c r="A33" t="s">
         <v>88</v>
       </c>
@@ -2823,7 +2890,7 @@
       <c r="F33" t="s">
         <v>53</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="1">
         <v>8009545212</v>
       </c>
       <c r="H33">
@@ -2847,10 +2914,10 @@
       <c r="N33">
         <v>3648</v>
       </c>
-      <c r="O33">
+      <c r="O33" s="3">
         <v>45779</v>
       </c>
-      <c r="P33">
+      <c r="P33" s="3">
         <v>56006</v>
       </c>
       <c r="Q33" t="s">
@@ -2864,151 +2931,192 @@
       </c>
       <c r="T33" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20">
+      <c r="A34" t="s">
+        <v>86</v>
+      </c>
+      <c r="B34" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D34" t="s">
+        <v>55</v>
+      </c>
+      <c r="E34" t="s">
+        <v>47</v>
+      </c>
+      <c r="F34" t="s">
+        <v>53</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H34">
+        <v>200000</v>
+      </c>
+      <c r="N34">
+        <v>2520</v>
+      </c>
+      <c r="O34" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="P34" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="S34" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:T33" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:T2 A3:M33 Q3:T33" numberStoredAsText="1"/>
   </ignoredErrors>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:7" ht="15.75">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B1" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F1" t="s">
         <v>1</v>
       </c>
       <c r="G1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75">
       <c r="A2" t="s">
         <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:7" ht="15.75">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75">
       <c r="A4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B5" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E6" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75">
       <c r="A7" t="s">
         <v>75</v>
       </c>
       <c r="B7" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D7" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75">
       <c r="D8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="E8" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75">
       <c r="D9" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E9" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -3022,9 +3130,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:13" ht="15.75">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -3065,27 +3173,27 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:13" ht="15.75">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
         <v>45</v>
       </c>
       <c r="D2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E2" t="s">
         <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="G2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H2">
         <v>500000</v>
@@ -3094,30 +3202,30 @@
         <v>6000</v>
       </c>
       <c r="J2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K2" t="s">
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="M2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.5">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="15.75">
       <c r="A3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E3" t="s">
         <v>47</v>
@@ -3126,7 +3234,7 @@
         <v>72</v>
       </c>
       <c r="G3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="H3" t="s">
         <v>1</v>
@@ -3135,7 +3243,7 @@
         <v>3600</v>
       </c>
       <c r="J3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="K3" t="s">
         <v>1</v>
@@ -3144,7 +3252,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: enforce idle logout across reloads, tab-close and PWA resume
The 30-min idle timer only ran while the tab stayed open; after closing/locking/
backgrounding, the 7-day cookie kept users logged in on return. Now last-activity
is persisted to localStorage and checked on mount and on focus/visibility change —
if away longer than 30 min, the user is logged out immediately on return.
</commit_message>
<xml_diff>
--- a/notion-import-templates/Insurance_Policies_Template.xlsx
+++ b/notion-import-templates/Insurance_Policies_Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="474" documentId="11_4902661BDEE849986904A2AD6474A91100A393FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81E4FB34-0875-44BA-8D1A-2426DBC56F5D}"/>
+  <xr:revisionPtr revIDLastSave="597" documentId="11_4902661BDEE849986904A2AD6474A91100A393FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{629F0596-6CED-488A-BDE5-EB11293112EC}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="821" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="225">
   <si>
     <t>Bill Morrisons — Insurance Policies Data Entry</t>
   </si>
@@ -74,6 +74,12 @@
     <t>CI Cover (MYR)</t>
   </si>
   <si>
+    <t>Early CI Cover (MYR)</t>
+  </si>
+  <si>
+    <t>Lady Cover</t>
+  </si>
+  <si>
     <t>PA Cover (MYR)</t>
   </si>
   <si>
@@ -132,6 +138,12 @@
   </si>
   <si>
     <t>Critical illness cover MYR (0 if same as SA)</t>
+  </si>
+  <si>
+    <t>Easrly CI cover MYR (0 if same as SA)</t>
+  </si>
+  <si>
+    <t>Lady cover MYR (0 if same as SA)</t>
   </si>
   <si>
     <t>Personal accident cover MYR (0 if same as SA)</t>
@@ -306,6 +318,9 @@
     <t>DORIS CHIEW JING TZE</t>
   </si>
   <si>
+    <t>🛡️ Life Cover, ⏸️ Waiver of Premium, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
+  </si>
+  <si>
     <t>0106809071</t>
   </si>
   <si>
@@ -321,13 +336,16 @@
     <t>CHAR CHEE LIM</t>
   </si>
   <si>
-    <t>🛡️ Life Cover, ♿ TPD, ❤️ Critical Illness (CI)</t>
+    <t>🛡️ Life Cover, ♿ TPD, 🌟 Early CI</t>
   </si>
   <si>
     <t>0106973912</t>
   </si>
   <si>
     <t>🛡️ Life Cover, ♿ TPD, 🏥 Medical, ⏸️ Waiver of Premium</t>
+  </si>
+  <si>
+    <t>🛡️ Life Cover, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
   </si>
   <si>
     <t>0104649955</t>
@@ -802,8 +820,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{69E5B004-7BF1-42CC-BE29-6E2C6D39DB56}" name="Table1" displayName="Table1" ref="N3:P33" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
-  <autoFilter ref="N3:P33" xr:uid="{69E5B004-7BF1-42CC-BE29-6E2C6D39DB56}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{69E5B004-7BF1-42CC-BE29-6E2C6D39DB56}" name="Table1" displayName="Table1" ref="P3:R33" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="P3:R33" xr:uid="{69E5B004-7BF1-42CC-BE29-6E2C6D39DB56}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{58D46586-83F1-4520-BB84-8DECA7EF760D}" name="Annual Premium (MYR)" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{0829D2FE-2862-4852-907C-03838995F0B3}" name="Commencement Date" dataDxfId="1"/>
@@ -1135,7 +1153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T61"/>
+  <dimension ref="A1:V61"/>
   <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="27.25" style="1" customWidth="1"/>
@@ -1147,20 +1165,20 @@
     <col min="7" max="7" width="12.625" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.25" style="1" customWidth="1"/>
     <col min="9" max="9" width="25.25" style="6" customWidth="1"/>
-    <col min="10" max="10" width="21" style="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5" style="1" customWidth="1"/>
-    <col min="12" max="12" width="35.75" style="1" customWidth="1"/>
-    <col min="13" max="13" width="29.375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.125" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="35.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9" style="1"/>
-    <col min="19" max="19" width="28.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="9" style="1"/>
+    <col min="10" max="12" width="21" style="1" customWidth="1"/>
+    <col min="13" max="13" width="20.5" style="1" customWidth="1"/>
+    <col min="14" max="14" width="35.75" style="1" customWidth="1"/>
+    <col min="15" max="15" width="29.375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="21.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="35.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9" style="1"/>
+    <col min="21" max="21" width="28.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:22">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1191,28 +1209,22 @@
       <c r="J1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R1" s="1" t="s">
+      <c r="O1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="S1" s="1" t="s">
@@ -1221,8 +1233,14 @@
       <c r="T1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:20">
+      <c r="U1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1253,28 +1271,22 @@
       <c r="J2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R2" s="1" t="s">
+      <c r="O2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="S2" s="1" t="s">
@@ -1283,8 +1295,14 @@
       <c r="T2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" ht="16.5">
+      <c r="U2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" ht="16.5">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1324,19 +1342,19 @@
       <c r="M3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="N3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="O3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="Q3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="R3" s="2" t="s">
         <v>20</v>
       </c>
       <c r="S3" s="1" t="s">
@@ -1345,90 +1363,102 @@
       <c r="T3" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:20" ht="32.25">
+      <c r="U3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" ht="32.25">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="O4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="N4" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="O4" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="P4" s="6" t="s">
         <v>40</v>
       </c>
+      <c r="Q4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="S4" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20">
+        <v>44</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22">
       <c r="A5" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="H5" s="1">
         <v>1000000</v>
@@ -1439,55 +1469,55 @@
       <c r="J5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L5" s="1">
-        <v>0</v>
-      </c>
       <c r="M5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N5" s="1">
+        <v>0</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P5" s="1">
         <v>5340</v>
       </c>
-      <c r="O5" s="3">
+      <c r="Q5" s="3">
         <v>43444</v>
       </c>
-      <c r="P5" s="3">
+      <c r="R5" s="3">
         <v>68281</v>
       </c>
-      <c r="Q5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S5" s="1" t="s">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="T5" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:20">
+      <c r="U5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22">
       <c r="A6" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G6" s="2">
         <v>6000739155</v>
@@ -1501,58 +1531,58 @@
       <c r="J6" s="1">
         <v>0</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L6" s="1">
-        <v>0</v>
-      </c>
       <c r="M6" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N6" s="1">
+        <v>0</v>
+      </c>
+      <c r="O6" s="1">
+        <v>200</v>
+      </c>
+      <c r="P6" s="1">
         <v>3204</v>
       </c>
-      <c r="O6" s="3">
+      <c r="Q6" s="3">
         <v>41968</v>
       </c>
-      <c r="P6" s="3">
+      <c r="R6" s="3">
         <v>68266</v>
       </c>
-      <c r="Q6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S6" s="1" t="s">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:20">
+      <c r="U6" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22">
       <c r="A7" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H7" s="1">
         <v>150000</v>
@@ -1563,58 +1593,58 @@
       <c r="J7" s="1">
         <v>0</v>
       </c>
-      <c r="K7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L7" s="1">
-        <v>0</v>
-      </c>
       <c r="M7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N7" s="1">
+        <v>0</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P7" s="1">
         <v>1200</v>
       </c>
-      <c r="O7" s="3">
+      <c r="Q7" s="3">
         <v>41291</v>
       </c>
-      <c r="P7" s="3">
+      <c r="R7" s="3">
         <v>68319</v>
       </c>
-      <c r="Q7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S7" s="1" t="s">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="T7" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:20">
+      <c r="U7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22">
       <c r="A8" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H8" s="1">
         <v>10000</v>
@@ -1625,58 +1655,58 @@
       <c r="J8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L8" s="1">
-        <v>0</v>
-      </c>
       <c r="M8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N8" s="1">
+        <v>0</v>
+      </c>
+      <c r="O8" s="1">
+        <v>150</v>
+      </c>
+      <c r="P8" s="1">
         <v>3960</v>
       </c>
-      <c r="O8" s="3">
+      <c r="Q8" s="3">
         <v>43517</v>
       </c>
-      <c r="P8" s="3">
+      <c r="R8" s="3">
         <v>60684</v>
       </c>
-      <c r="Q8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R8" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S8" s="1" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="T8" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:20">
+      <c r="U8" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="V8" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22">
       <c r="A9" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H9" s="1">
         <v>50000</v>
@@ -1687,55 +1717,55 @@
       <c r="J9" s="1">
         <v>150000</v>
       </c>
-      <c r="K9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L9" s="1">
-        <v>0</v>
-      </c>
       <c r="M9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N9" s="1">
+        <v>0</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P9" s="1">
         <v>1800</v>
       </c>
-      <c r="O9" s="3">
+      <c r="Q9" s="3">
         <v>42252</v>
       </c>
-      <c r="P9" s="3">
+      <c r="R9" s="3">
         <v>65263</v>
       </c>
-      <c r="Q9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R9" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S9" s="1" t="s">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="T9" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:20">
+      <c r="U9" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="V9" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22">
       <c r="A10" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G10" s="2">
         <v>8009558744</v>
@@ -1749,55 +1779,55 @@
       <c r="J10" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L10" s="1">
-        <v>0</v>
-      </c>
       <c r="M10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N10" s="1">
+        <v>0</v>
+      </c>
+      <c r="O10" s="1">
+        <v>300</v>
+      </c>
+      <c r="P10" s="1">
         <v>4020</v>
       </c>
-      <c r="O10" s="3">
+      <c r="Q10" s="3">
         <v>45783</v>
       </c>
-      <c r="P10" s="3">
+      <c r="R10" s="3">
         <v>54184</v>
       </c>
-      <c r="Q10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R10" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S10" s="1" t="s">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:20">
+      <c r="U10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22">
       <c r="A11" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G11" s="2">
         <v>8001890884</v>
@@ -1805,61 +1835,61 @@
       <c r="H11" s="1">
         <v>100000</v>
       </c>
-      <c r="I11" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>1</v>
+      <c r="I11" s="6">
+        <v>0</v>
+      </c>
+      <c r="J11" s="1">
+        <v>0</v>
       </c>
       <c r="M11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N11" s="1">
+        <v>0</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P11" s="1">
         <v>1800</v>
       </c>
-      <c r="O11" s="3">
+      <c r="Q11" s="3">
         <v>43309</v>
       </c>
-      <c r="P11" s="3">
+      <c r="R11" s="3">
         <v>79103</v>
       </c>
-      <c r="Q11" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="R11" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S11" s="1" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="T11" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:20">
+      <c r="U11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V11" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22">
       <c r="A12" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G12" s="2">
         <v>8010673726</v>
@@ -1867,61 +1897,61 @@
       <c r="H12" s="1">
         <v>5000</v>
       </c>
-      <c r="I12" s="6" t="s">
-        <v>1</v>
+      <c r="I12" s="6">
+        <v>0</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L12" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N12" s="1">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1">
+        <v>200</v>
+      </c>
+      <c r="P12" s="1">
         <v>1896</v>
       </c>
-      <c r="O12" s="3">
+      <c r="Q12" s="3">
         <v>46092</v>
       </c>
-      <c r="P12" s="3">
+      <c r="R12" s="3">
         <v>71660</v>
       </c>
-      <c r="Q12" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="R12" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S12" s="1" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="T12" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:20">
+      <c r="U12" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V12" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
       <c r="A13" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G13" s="2">
         <v>8010673637</v>
@@ -1929,61 +1959,61 @@
       <c r="H13" s="1">
         <v>5000</v>
       </c>
-      <c r="I13" s="6" t="s">
-        <v>1</v>
+      <c r="I13" s="6">
+        <v>0</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N13" s="1">
+        <v>0</v>
+      </c>
+      <c r="O13" s="1">
+        <v>200</v>
+      </c>
+      <c r="P13" s="1">
         <v>5604</v>
       </c>
-      <c r="O13" s="3">
+      <c r="Q13" s="3">
         <v>46092</v>
       </c>
-      <c r="P13" s="3">
+      <c r="R13" s="3">
         <v>57415</v>
       </c>
-      <c r="Q13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R13" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S13" s="1" t="s">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="T13" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:20">
+      <c r="U13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="V13" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22">
       <c r="A14" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G14" s="2">
         <v>6001000871</v>
@@ -1991,61 +2021,61 @@
       <c r="H14" s="1">
         <v>200000</v>
       </c>
-      <c r="I14" s="6" t="s">
-        <v>1</v>
+      <c r="I14" s="6">
+        <v>0</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M14" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N14" s="1">
+        <v>0</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P14" s="1">
         <v>2400</v>
       </c>
-      <c r="O14" s="3">
+      <c r="Q14" s="3">
         <v>42142</v>
       </c>
-      <c r="P14" s="3">
+      <c r="R14" s="3">
         <v>64788</v>
       </c>
-      <c r="Q14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R14" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S14" s="1" t="s">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:20">
+      <c r="U14" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="V14" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22">
       <c r="A15" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G15" s="2">
         <v>35438762</v>
@@ -2059,55 +2089,55 @@
       <c r="J15" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M15" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P15" s="1">
         <v>7392</v>
       </c>
-      <c r="O15" s="3">
+      <c r="Q15" s="3">
         <v>43344</v>
       </c>
-      <c r="P15" s="3">
+      <c r="R15" s="3">
         <v>64529</v>
       </c>
-      <c r="Q15" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R15" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S15" s="1" t="s">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="T15" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:20">
+      <c r="U15" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="V15" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22">
       <c r="A16" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="G16" s="2">
         <v>31359163</v>
@@ -2121,55 +2151,55 @@
       <c r="J16" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M16" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P16" s="1">
         <v>5868.6</v>
       </c>
-      <c r="O16" s="3">
+      <c r="Q16" s="3">
         <v>45292</v>
       </c>
-      <c r="P16" s="3">
+      <c r="R16" s="3">
         <v>57346</v>
       </c>
-      <c r="Q16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R16" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S16" s="1" t="s">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="T16" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:20">
+      <c r="U16" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V16" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22">
       <c r="A17" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G17" s="2">
         <v>35439348</v>
@@ -2183,55 +2213,55 @@
       <c r="J17" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L17" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M17" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P17" s="1">
         <v>6924</v>
       </c>
-      <c r="O17" s="3">
+      <c r="Q17" s="3">
         <v>43344</v>
       </c>
-      <c r="P17" s="3">
+      <c r="R17" s="3">
         <v>66355</v>
       </c>
-      <c r="Q17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R17" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S17" s="1" t="s">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="T17" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:20">
+      <c r="U17" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="V17" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22">
       <c r="A18" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G18" s="2">
         <v>6000739226</v>
@@ -2239,61 +2269,61 @@
       <c r="H18" s="1">
         <v>100000</v>
       </c>
-      <c r="I18" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>1</v>
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
+        <v>150000</v>
       </c>
       <c r="M18" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P18" s="1">
         <v>2400</v>
       </c>
-      <c r="O18" s="3">
+      <c r="Q18" s="3">
         <v>41969</v>
       </c>
-      <c r="P18" s="3">
+      <c r="R18" s="3">
         <v>66806</v>
       </c>
-      <c r="Q18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S18" s="1" t="s">
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="T18" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:20">
+      <c r="U18" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="V18" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22">
       <c r="A19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="C19" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G19" s="2">
         <v>8010673612</v>
@@ -2301,61 +2331,61 @@
       <c r="H19" s="1">
         <v>5000</v>
       </c>
-      <c r="I19" s="6" t="s">
-        <v>1</v>
+      <c r="I19" s="6">
+        <v>0</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M19" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <v>200</v>
+      </c>
+      <c r="P19" s="1">
         <v>4200</v>
       </c>
-      <c r="O19" s="3">
+      <c r="Q19" s="3">
         <v>46092</v>
       </c>
-      <c r="P19" s="3">
+      <c r="R19" s="3">
         <v>59241</v>
       </c>
-      <c r="Q19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S19" s="1" t="s">
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="T19" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:20">
+      <c r="U19" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="V19" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22">
       <c r="A20" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G20" s="2">
         <v>8010751037</v>
@@ -2363,61 +2393,61 @@
       <c r="H20" s="1">
         <v>5000</v>
       </c>
-      <c r="I20" s="6" t="s">
-        <v>1</v>
+      <c r="I20" s="6">
+        <v>0</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K20" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M20" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N20" s="1">
+        <v>0</v>
+      </c>
+      <c r="O20" s="1">
+        <v>200</v>
+      </c>
+      <c r="P20" s="1">
         <v>1824</v>
       </c>
-      <c r="O20" s="3">
+      <c r="Q20" s="3">
         <v>46111</v>
       </c>
-      <c r="P20" s="3">
+      <c r="R20" s="3">
         <v>69850</v>
       </c>
-      <c r="Q20" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="R20" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S20" s="1" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="T20" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:20">
+      <c r="U20" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V20" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22">
       <c r="A21" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G21" s="2">
         <v>8010750874</v>
@@ -2425,58 +2455,58 @@
       <c r="H21" s="1">
         <v>5000</v>
       </c>
-      <c r="I21" s="6" t="s">
-        <v>1</v>
+      <c r="I21" s="6">
+        <v>0</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K21" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M21" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N21" s="1">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1">
+        <v>200</v>
+      </c>
+      <c r="P21" s="1">
         <v>4248</v>
       </c>
-      <c r="O21" s="3">
+      <c r="Q21" s="3">
         <v>46111</v>
       </c>
-      <c r="P21" s="3">
+      <c r="R21" s="3">
         <v>60719</v>
       </c>
-      <c r="R21" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="S21" s="1" t="s">
-        <v>80</v>
-      </c>
       <c r="T21" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:20">
+      <c r="U21" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="V21" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22">
       <c r="A22" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G22" s="2">
         <v>8010750804</v>
@@ -2484,61 +2514,61 @@
       <c r="H22" s="1">
         <v>5000</v>
       </c>
-      <c r="I22" s="6" t="s">
-        <v>1</v>
+      <c r="I22" s="6">
+        <v>0</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K22" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M22" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N22" s="1">
+        <v>0</v>
+      </c>
+      <c r="O22" s="1">
+        <v>200</v>
+      </c>
+      <c r="P22" s="1">
         <v>1848</v>
       </c>
-      <c r="O22" s="3">
+      <c r="Q22" s="3">
         <v>46111</v>
       </c>
-      <c r="P22" s="3">
+      <c r="R22" s="3">
         <v>68389</v>
       </c>
-      <c r="Q22" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="R22" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S22" s="1" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="T22" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:20">
+      <c r="U22" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V22" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22">
       <c r="A23" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G23" s="2">
         <v>8003557527</v>
@@ -2546,61 +2576,61 @@
       <c r="H23" s="1">
         <v>500000</v>
       </c>
-      <c r="I23" s="6" t="s">
-        <v>1</v>
+      <c r="I23" s="6">
+        <v>0</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M23" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N23" s="1">
+        <v>0</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P23" s="1">
         <v>1800</v>
       </c>
-      <c r="O23" s="3">
+      <c r="Q23" s="3">
         <v>43859</v>
       </c>
-      <c r="P23" s="3">
+      <c r="R23" s="3">
         <v>54816</v>
       </c>
-      <c r="Q23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R23" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S23" s="1" t="s">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="T23" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:20">
+      <c r="U23" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="V23" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22">
       <c r="A24" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G24" s="2">
         <v>6001564581</v>
@@ -2608,61 +2638,61 @@
       <c r="H24" s="1">
         <v>100000</v>
       </c>
-      <c r="I24" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K24" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L24" s="1" t="s">
-        <v>1</v>
+      <c r="I24" s="6">
+        <v>0</v>
+      </c>
+      <c r="J24" s="1">
+        <v>0</v>
       </c>
       <c r="M24" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N24" s="1">
+        <v>0</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P24" s="1">
         <v>1800</v>
       </c>
-      <c r="O24" s="3">
+      <c r="Q24" s="3">
         <v>42621</v>
       </c>
-      <c r="P24" s="3">
+      <c r="R24" s="3">
         <v>68188</v>
       </c>
-      <c r="Q24" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R24" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S24" s="1" t="s">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="T24" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:20">
+      <c r="U24" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="V24" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22">
       <c r="A25" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G25" s="2">
         <v>8003219923</v>
@@ -2670,61 +2700,61 @@
       <c r="H25" s="1">
         <v>1000000</v>
       </c>
-      <c r="I25" s="6" t="s">
-        <v>1</v>
+      <c r="I25" s="6">
+        <v>0</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M25" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N25" s="1">
+        <v>0</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P25" s="1">
         <v>2232</v>
       </c>
-      <c r="O25" s="3">
+      <c r="Q25" s="3">
         <v>43752</v>
       </c>
-      <c r="P25" s="3">
+      <c r="R25" s="3">
         <v>51423</v>
       </c>
-      <c r="Q25" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R25" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S25" s="1" t="s">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="T25" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:20">
+      <c r="U25" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="V25" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22">
       <c r="A26" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G26" s="2">
         <v>8001036225</v>
@@ -2732,58 +2762,61 @@
       <c r="H26" s="1">
         <v>100000</v>
       </c>
-      <c r="I26" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>1</v>
+      <c r="I26" s="6">
+        <v>0</v>
+      </c>
+      <c r="J26" s="1">
+        <v>0</v>
       </c>
       <c r="M26" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N26" s="1">
+        <v>0</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P26" s="1">
         <v>1200</v>
       </c>
-      <c r="O26" s="3">
+      <c r="Q26" s="3">
         <v>42993</v>
       </c>
-      <c r="P26" s="3">
+      <c r="R26" s="3">
         <v>79152</v>
       </c>
-      <c r="Q26" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="R26" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S26" s="1" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="T26" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:20">
+      <c r="U26" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V26" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22">
       <c r="A27" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G27" s="2">
         <v>8005353726</v>
@@ -2791,371 +2824,375 @@
       <c r="H27" s="1">
         <v>100000</v>
       </c>
-      <c r="I27" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>1</v>
+      <c r="I27" s="6">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1">
+        <v>0</v>
       </c>
       <c r="M27" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N27" s="1">
+        <v>0</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P27" s="1">
         <v>1200</v>
       </c>
-      <c r="O27" s="3">
+      <c r="Q27" s="3">
         <v>44447</v>
       </c>
-      <c r="P27" s="3">
+      <c r="R27" s="3">
         <v>75857</v>
       </c>
-      <c r="Q27" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="R27" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S27" s="1" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="T27" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:20">
+      <c r="U27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V27" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22">
       <c r="A28" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H28" s="1">
         <v>100000</v>
       </c>
-      <c r="I28" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L28" s="1" t="s">
-        <v>1</v>
+      <c r="I28" s="6">
+        <v>0</v>
+      </c>
+      <c r="J28" s="1">
+        <v>0</v>
       </c>
       <c r="M28" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N28" s="1">
+        <v>0</v>
+      </c>
+      <c r="O28" s="1">
+        <v>200</v>
+      </c>
+      <c r="P28" s="1">
         <v>2304</v>
       </c>
-      <c r="O28" s="3">
+      <c r="Q28" s="3">
         <v>41269</v>
       </c>
-      <c r="P28" s="3">
+      <c r="R28" s="3">
         <v>67932</v>
       </c>
-      <c r="Q28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R28" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S28" s="1" t="s">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="T28" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:20">
+      <c r="U28" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="V28" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22">
       <c r="A29" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H29" s="1">
         <v>100000</v>
       </c>
-      <c r="I29" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L29" s="1" t="s">
-        <v>1</v>
+      <c r="I29" s="6">
+        <v>0</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0</v>
       </c>
       <c r="M29" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N29" s="1">
+        <v>0</v>
+      </c>
+      <c r="O29" s="1">
+        <v>200</v>
+      </c>
+      <c r="P29" s="1">
         <v>3744</v>
       </c>
-      <c r="O29" s="3">
+      <c r="Q29" s="3">
         <v>40704</v>
       </c>
-      <c r="P29" s="3">
+      <c r="R29" s="3">
         <v>68098</v>
       </c>
-      <c r="Q29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R29" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S29" s="1" t="s">
-        <v>89</v>
+        <v>1</v>
       </c>
       <c r="T29" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:20">
+      <c r="U29" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="V29" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22">
       <c r="A30" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H30" s="1">
         <v>300000</v>
       </c>
-      <c r="I30" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K30" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L30" s="1" t="s">
-        <v>1</v>
-      </c>
+      <c r="I30" s="6">
+        <v>0</v>
+      </c>
+      <c r="J30" s="1">
+        <v>100000</v>
+      </c>
+      <c r="K30" s="9">
+        <v>200000</v>
+      </c>
+      <c r="L30" s="9"/>
       <c r="M30" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N30" s="1">
+        <v>0</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P30" s="1">
         <v>2400</v>
       </c>
-      <c r="O30" s="3">
+      <c r="Q30" s="3">
         <v>41479</v>
       </c>
-      <c r="P30" s="3">
+      <c r="R30" s="3">
         <v>68142</v>
       </c>
-      <c r="Q30" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R30" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S30" s="1" t="s">
-        <v>89</v>
+        <v>1</v>
       </c>
       <c r="T30" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:20">
+      <c r="U30" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="V30" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22">
       <c r="A31" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="H31" s="1">
         <v>55000</v>
       </c>
-      <c r="I31" s="6" t="s">
-        <v>1</v>
+      <c r="I31" s="6">
+        <v>0</v>
       </c>
       <c r="J31" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K31" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M31" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N31" s="1">
+        <v>0</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P31" s="1">
         <v>1200</v>
       </c>
-      <c r="O31" s="3">
+      <c r="Q31" s="3">
         <v>40145</v>
       </c>
-      <c r="P31" s="3">
+      <c r="R31" s="3">
         <v>67173</v>
       </c>
-      <c r="Q31" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R31" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S31" s="1" t="s">
-        <v>94</v>
+        <v>1</v>
       </c>
       <c r="T31" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:20">
+      <c r="U31" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="V31" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22">
       <c r="A32" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H32" s="1">
         <v>10000</v>
       </c>
-      <c r="I32" s="6" t="s">
-        <v>1</v>
+      <c r="I32" s="6">
+        <v>0</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K32" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L32" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="M32" s="1" t="s">
-        <v>1</v>
+      <c r="K32" s="1">
+        <v>70000</v>
       </c>
       <c r="N32" s="1">
+        <v>0</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P32" s="1">
         <v>1200</v>
       </c>
-      <c r="O32" s="3">
+      <c r="Q32" s="3">
         <v>41535</v>
       </c>
-      <c r="P32" s="3">
+      <c r="R32" s="3">
         <v>67102</v>
       </c>
-      <c r="Q32" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R32" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S32" s="1" t="s">
-        <v>94</v>
+        <v>1</v>
       </c>
       <c r="T32" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:20">
+      <c r="U32" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="V32" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22">
       <c r="A33" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G33" s="2">
         <v>8009545212</v>
@@ -3163,137 +3200,149 @@
       <c r="H33" s="1">
         <v>5000</v>
       </c>
-      <c r="I33" s="6" t="s">
-        <v>1</v>
+      <c r="I33" s="6">
+        <v>0</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L33" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="M33" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N33" s="1">
+        <v>0</v>
+      </c>
+      <c r="O33" s="1">
+        <v>300</v>
+      </c>
+      <c r="P33" s="1">
         <v>3648</v>
       </c>
-      <c r="O33" s="3">
+      <c r="Q33" s="3">
         <v>45779</v>
       </c>
-      <c r="P33" s="3">
+      <c r="R33" s="3">
         <v>56006</v>
       </c>
-      <c r="Q33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="R33" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="S33" s="1" t="s">
-        <v>94</v>
+        <v>1</v>
       </c>
       <c r="T33" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:20">
+      <c r="U33" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="V33" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22">
       <c r="A34" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>55</v>
+        <v>103</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="H34" s="1">
         <v>200000</v>
       </c>
+      <c r="I34" s="6">
+        <v>0</v>
+      </c>
+      <c r="J34" s="1">
+        <v>150000</v>
+      </c>
+      <c r="K34" s="1">
+        <v>150000</v>
+      </c>
       <c r="N34" s="1">
+        <v>0</v>
+      </c>
+      <c r="P34" s="1">
         <v>2520</v>
       </c>
-      <c r="O34" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="P34" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="S34" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20">
+      <c r="Q34" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="R34" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="U34" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22">
       <c r="A35" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H35" s="1">
         <v>100000</v>
       </c>
-      <c r="N35" s="1">
+      <c r="P35" s="1">
         <v>2760</v>
       </c>
-      <c r="O35" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="P35" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="S35" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20">
+      <c r="Q35" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="R35" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="U35" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22">
       <c r="A36" s="1" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G36" s="2">
         <v>8000474682</v>
@@ -3301,37 +3350,46 @@
       <c r="H36" s="1">
         <v>50000</v>
       </c>
+      <c r="I36" s="6">
+        <v>0</v>
+      </c>
+      <c r="K36" s="1">
+        <v>100000</v>
+      </c>
       <c r="N36" s="1">
+        <v>0</v>
+      </c>
+      <c r="P36" s="1">
         <v>1800</v>
       </c>
-      <c r="O36" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="P36" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q36" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="37" spans="1:20">
+      <c r="Q36" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="R36" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="S36" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22">
       <c r="A37" s="1" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G37" s="2">
         <v>8000474701</v>
@@ -3339,40 +3397,49 @@
       <c r="H37" s="1">
         <v>50000</v>
       </c>
+      <c r="I37" s="6">
+        <v>0</v>
+      </c>
+      <c r="K37" s="1">
+        <v>100000</v>
+      </c>
       <c r="N37" s="1">
+        <v>0</v>
+      </c>
+      <c r="P37" s="1">
         <v>1800</v>
       </c>
-      <c r="O37" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="P37" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q37" s="1" t="s">
-        <v>108</v>
+      <c r="Q37" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="R37" s="3" t="s">
+        <v>116</v>
       </c>
       <c r="S37" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20">
+        <v>114</v>
+      </c>
+      <c r="U37" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22">
       <c r="A38" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>105</v>
-      </c>
       <c r="E38" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G38" s="2">
         <v>8000474735</v>
@@ -3380,40 +3447,49 @@
       <c r="H38" s="1">
         <v>50000</v>
       </c>
+      <c r="I38" s="6">
+        <v>0</v>
+      </c>
+      <c r="K38" s="1">
+        <v>100000</v>
+      </c>
       <c r="N38" s="1">
+        <v>0</v>
+      </c>
+      <c r="P38" s="1">
         <v>1800</v>
       </c>
-      <c r="O38" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="P38" s="3" t="s">
+      <c r="Q38" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="Q38" s="1" t="s">
-        <v>108</v>
+      <c r="R38" s="3" t="s">
+        <v>118</v>
       </c>
       <c r="S38" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" ht="64.5">
+        <v>114</v>
+      </c>
+      <c r="U38" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" ht="64.5">
       <c r="A39" s="1" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G39" s="2">
         <v>8000319947</v>
@@ -3421,37 +3497,49 @@
       <c r="H39" s="1">
         <v>110000</v>
       </c>
+      <c r="I39" s="6">
+        <v>0</v>
+      </c>
+      <c r="K39" s="1">
+        <v>100000</v>
+      </c>
       <c r="N39" s="1">
+        <v>0</v>
+      </c>
+      <c r="O39" s="1">
+        <v>200</v>
+      </c>
+      <c r="P39" s="1">
         <v>7608</v>
       </c>
-      <c r="O39" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="P39" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="S39" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="40" spans="1:20">
+      <c r="Q39" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="R39" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="U39" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22">
       <c r="A40" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G40" s="2">
         <v>8001136733</v>
@@ -3459,75 +3547,93 @@
       <c r="H40" s="1">
         <v>100000</v>
       </c>
+      <c r="I40" s="6">
+        <v>0</v>
+      </c>
+      <c r="J40" s="1">
+        <v>0</v>
+      </c>
       <c r="N40" s="1">
+        <v>0</v>
+      </c>
+      <c r="O40" s="1">
+        <v>200</v>
+      </c>
+      <c r="P40" s="1">
         <v>2892</v>
       </c>
-      <c r="O40" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="P40" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="Q40" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="41" spans="1:20">
+      <c r="Q40" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="R40" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="S40" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22">
       <c r="A41" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G41" s="2">
         <v>6000914783</v>
       </c>
       <c r="H41" s="1">
-        <v>41400</v>
+        <v>414000</v>
+      </c>
+      <c r="I41" s="6">
+        <v>0</v>
       </c>
       <c r="N41" s="1">
+        <v>0</v>
+      </c>
+      <c r="P41" s="1">
         <v>2400</v>
       </c>
-      <c r="O41" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="P41" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="S41" s="1" t="s">
+      <c r="Q41" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="R41" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="U41" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22">
+      <c r="A42" s="1" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="42" spans="1:20">
-      <c r="A42" s="1" t="s">
-        <v>117</v>
-      </c>
       <c r="B42" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G42" s="2">
         <v>8009554653</v>
@@ -3535,37 +3641,46 @@
       <c r="H42" s="1">
         <v>5000</v>
       </c>
+      <c r="I42" s="6">
+        <v>0</v>
+      </c>
       <c r="N42" s="1">
+        <v>0</v>
+      </c>
+      <c r="O42" s="1">
+        <v>300</v>
+      </c>
+      <c r="P42" s="1">
         <v>1764</v>
       </c>
-      <c r="O42" s="3">
+      <c r="Q42" s="3">
         <v>45782</v>
       </c>
-      <c r="P42" s="3">
+      <c r="R42" s="3">
         <v>68427</v>
       </c>
-      <c r="Q42" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="43" spans="1:20" ht="16.5">
+      <c r="S42" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" ht="16.5">
       <c r="A43" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G43" s="2">
         <v>8006861955</v>
@@ -3573,113 +3688,137 @@
       <c r="H43" s="1">
         <v>500000</v>
       </c>
+      <c r="I43" s="6">
+        <v>0</v>
+      </c>
       <c r="N43" s="1">
+        <v>0</v>
+      </c>
+      <c r="P43" s="1">
         <v>2499.96</v>
       </c>
-      <c r="O43" s="3">
+      <c r="Q43" s="3">
         <v>45200</v>
       </c>
-      <c r="P43" s="3">
+      <c r="R43" s="3">
         <v>61271</v>
       </c>
-      <c r="S43" s="6" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="44" spans="1:20" ht="48.75">
+      <c r="U43" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" ht="48.75">
       <c r="A44" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="H44" s="1">
         <v>100000</v>
       </c>
+      <c r="I44" s="6">
+        <v>0</v>
+      </c>
+      <c r="J44" s="1">
+        <v>0</v>
+      </c>
       <c r="N44" s="1">
+        <v>0</v>
+      </c>
+      <c r="P44" s="1">
         <v>1800</v>
       </c>
-      <c r="O44" s="7">
+      <c r="Q44" s="7">
         <v>40057</v>
       </c>
-      <c r="P44" s="3">
+      <c r="R44" s="3">
         <v>68181</v>
       </c>
-      <c r="S44" s="6" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="45" spans="1:20" ht="32.25">
+      <c r="U44" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" ht="32.25">
       <c r="A45" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="H45" s="1">
         <v>160000</v>
       </c>
+      <c r="I45" s="6">
+        <v>0</v>
+      </c>
+      <c r="J45" s="1">
+        <v>0</v>
+      </c>
       <c r="N45" s="1">
+        <v>0</v>
+      </c>
+      <c r="P45" s="1">
         <v>1200</v>
       </c>
-      <c r="O45" s="3" t="s">
+      <c r="Q45" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="R45" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="U45" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22">
+      <c r="A46" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="P45" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="S45" s="6" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="46" spans="1:20">
-      <c r="A46" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="B46" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G46" s="2">
         <v>8010004645</v>
@@ -3687,113 +3826,137 @@
       <c r="H46" s="1">
         <v>5000</v>
       </c>
+      <c r="I46" s="6">
+        <v>0</v>
+      </c>
       <c r="N46" s="1">
+        <v>0</v>
+      </c>
+      <c r="O46" s="1">
+        <v>200</v>
+      </c>
+      <c r="P46" s="1">
         <v>3000</v>
       </c>
-      <c r="O46" s="3">
+      <c r="Q46" s="3">
         <v>45879</v>
       </c>
-      <c r="P46" s="3">
+      <c r="R46" s="3">
         <v>57202</v>
       </c>
-      <c r="S46" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="47" spans="1:20">
+      <c r="U46" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22">
       <c r="A47" s="1" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H47" s="1">
         <v>1000000</v>
       </c>
-      <c r="N47" s="1">
+      <c r="P47" s="1">
         <v>5340</v>
       </c>
-      <c r="O47" s="3">
+      <c r="Q47" s="3">
         <v>43378</v>
       </c>
-      <c r="P47" s="3">
+      <c r="R47" s="3">
         <v>68215</v>
       </c>
-      <c r="S47" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="48" spans="1:20">
+      <c r="U47" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22">
       <c r="A48" s="1" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="H48" s="1">
         <v>100000</v>
       </c>
+      <c r="I48" s="6">
+        <v>0</v>
+      </c>
+      <c r="J48" s="1">
+        <v>0</v>
+      </c>
+      <c r="L48" s="1">
+        <v>50000</v>
+      </c>
       <c r="N48" s="1">
+        <v>0</v>
+      </c>
+      <c r="O48" s="1">
+        <v>200</v>
+      </c>
+      <c r="P48" s="1">
         <v>4368</v>
       </c>
-      <c r="O48" s="3">
+      <c r="Q48" s="3">
         <v>40975</v>
       </c>
-      <c r="P48" s="3">
+      <c r="R48" s="3">
         <v>68368</v>
       </c>
-      <c r="S48" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="49" spans="1:19" ht="32.25">
+      <c r="U48" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="49" spans="1:21" ht="32.25">
       <c r="A49" s="1" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G49" s="2">
         <v>6001549235</v>
@@ -3801,113 +3964,119 @@
       <c r="H49" s="1">
         <v>600000</v>
       </c>
+      <c r="I49" s="6">
+        <v>0</v>
+      </c>
       <c r="N49" s="1">
+        <v>0</v>
+      </c>
+      <c r="P49" s="1">
         <v>1440</v>
       </c>
-      <c r="O49" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="P49" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="S49" s="6" t="s">
+      <c r="Q49" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="R49" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="U49" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" ht="32.25">
+      <c r="A50" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="50" spans="1:19" ht="32.25">
-      <c r="A50" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="B50" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="H50" s="1">
         <v>50000</v>
       </c>
-      <c r="N50" s="1">
+      <c r="P50" s="1">
         <v>1500</v>
       </c>
-      <c r="O50" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="P50" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="S50" s="6" t="s">
+      <c r="Q50" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="R50" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="U50" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21">
+      <c r="A51" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="51" spans="1:19">
-      <c r="A51" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="B51" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="H51" s="1">
         <v>150000</v>
       </c>
-      <c r="N51" s="1">
+      <c r="P51" s="1">
         <v>1200</v>
       </c>
-      <c r="O51" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="P51" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="S51" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="52" spans="1:19" ht="32.25">
+      <c r="Q51" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="R51" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="U51" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="52" spans="1:21" ht="32.25">
       <c r="A52" s="1" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G52" s="2">
         <v>8005001007</v>
@@ -3915,37 +4084,37 @@
       <c r="H52" s="1">
         <v>600000</v>
       </c>
-      <c r="N52" s="1">
+      <c r="P52" s="1">
         <v>2400</v>
       </c>
-      <c r="O52" s="3">
+      <c r="Q52" s="3">
         <v>44413</v>
       </c>
-      <c r="P52" s="3">
+      <c r="R52" s="3">
         <v>61214</v>
       </c>
-      <c r="S52" s="6" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19">
+      <c r="U52" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21">
       <c r="A53" s="1" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G53" s="2">
         <v>8009518746</v>
@@ -3953,37 +4122,37 @@
       <c r="H53" s="1">
         <v>5000</v>
       </c>
-      <c r="N53" s="1">
+      <c r="P53" s="1">
         <v>3132</v>
       </c>
-      <c r="O53" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="P53" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="S53" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="54" spans="1:19">
+      <c r="Q53" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="R53" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="U53" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21">
       <c r="A54" s="1" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G54" s="2">
         <v>8005001052</v>
@@ -3991,37 +4160,37 @@
       <c r="H54" s="1">
         <v>1500000</v>
       </c>
-      <c r="N54" s="1">
+      <c r="P54" s="1">
         <v>6000</v>
       </c>
-      <c r="O54" s="3">
+      <c r="Q54" s="3">
         <v>44201</v>
       </c>
-      <c r="P54" s="3">
+      <c r="R54" s="3">
         <v>56984</v>
       </c>
-      <c r="S54" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="55" spans="1:19" ht="16.5">
+      <c r="U54" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" ht="16.5">
       <c r="A55" s="1" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G55" s="2">
         <v>6001512162</v>
@@ -4029,37 +4198,37 @@
       <c r="H55" s="1">
         <v>100000</v>
       </c>
-      <c r="N55" s="1">
+      <c r="P55" s="1">
         <v>1800</v>
       </c>
-      <c r="O55" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="P55" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="S55" s="6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="56" spans="1:19">
+      <c r="Q55" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="R55" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="U55" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21">
       <c r="A56" s="1" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G56" s="2">
         <v>8002084775</v>
@@ -4067,40 +4236,40 @@
       <c r="H56" s="1">
         <v>100000</v>
       </c>
-      <c r="N56" s="1">
+      <c r="P56" s="1">
         <v>12000</v>
       </c>
-      <c r="O56" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="P56" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="S56" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="57" spans="1:19">
+      <c r="Q56" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="R56" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="U56" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="57" spans="1:21">
       <c r="A57" s="1" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="H57" s="1">
         <v>100000</v>
@@ -4111,113 +4280,115 @@
       <c r="J57" s="9">
         <v>200000</v>
       </c>
-      <c r="L57" s="1">
-        <v>0</v>
-      </c>
+      <c r="K57" s="9"/>
+      <c r="L57" s="9"/>
       <c r="N57" s="1">
+        <v>0</v>
+      </c>
+      <c r="P57" s="1">
         <v>2400</v>
       </c>
-      <c r="O57" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="P57" s="3" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="58" spans="1:19" ht="32.25">
+      <c r="Q57" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="R57" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="58" spans="1:21" ht="32.25">
       <c r="A58" s="1" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="H58" s="1">
         <v>100000</v>
       </c>
-      <c r="N58" s="1">
+      <c r="P58" s="1">
         <v>1800</v>
       </c>
-      <c r="O58" s="3">
+      <c r="Q58" s="3">
         <v>40158</v>
       </c>
-      <c r="P58" s="3">
+      <c r="R58" s="3">
         <v>68282</v>
       </c>
-      <c r="S58" s="6" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="59" spans="1:19" ht="32.25">
+      <c r="U58" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" ht="32.25">
       <c r="A59" s="1" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="H59" s="1">
         <v>150000</v>
       </c>
-      <c r="N59" s="1">
+      <c r="P59" s="1">
         <v>3000</v>
       </c>
-      <c r="O59" s="3">
+      <c r="Q59" s="3">
         <v>41156</v>
       </c>
-      <c r="P59" s="3">
+      <c r="R59" s="3">
         <v>68184</v>
       </c>
-      <c r="S59" s="6" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="60" spans="1:19">
+      <c r="U59" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="60" spans="1:21">
       <c r="A60" s="1" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G60" s="2">
         <v>8010660964</v>
@@ -4225,58 +4396,58 @@
       <c r="H60" s="1">
         <v>5000</v>
       </c>
-      <c r="N60" s="1">
+      <c r="P60" s="1">
         <v>3672</v>
       </c>
-      <c r="O60" s="3">
+      <c r="Q60" s="3">
         <v>46089</v>
       </c>
-      <c r="P60" s="3">
+      <c r="R60" s="3">
         <v>61064</v>
       </c>
-      <c r="S60" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="61" spans="1:19">
+      <c r="U60" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="61" spans="1:21">
       <c r="A61" s="1" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="H61" s="1">
         <v>500000</v>
       </c>
-      <c r="N61" s="1">
+      <c r="P61" s="1">
         <v>1800</v>
       </c>
-      <c r="O61" s="3">
+      <c r="Q61" s="3">
         <v>44409</v>
       </c>
-      <c r="P61" s="3">
+      <c r="R61" s="3">
         <v>56097</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:T2 A3:M3 Q3:T10 A28:M33 B26:K26 M26 A23:M25 B22:M22 Q23:T25 R20:T20 A21:M21 B20:M20 R21:T21 R22:T22 Q28:T33 R26:T26 B27:M27 R27:T27 Q13:T19 R11:T11 A13:M19 B11:M11 B12:M12 R12:T12 A10:H10 A5 C5:H5 A4:J4 M5 J5:K5 A6:H6 K6 M6 A7:H7 M7 K7 A8:H8 M8 J8:K8 A9:H9 K9 M9 J10:K10 M10" numberStoredAsText="1"/>
+    <ignoredError sqref="M1:V2 M3:O3 S3:V10 M33 B26:H26 O26 A25:H25 B22:H22 S23:V25 T20:V20 A21:H21 B20:H20 T21:V21 T22:V22 S28:V33 T26:V26 B27:H27 T27:V27 S13:V19 T11:V11 M15:O17 B11:H11 B12:H12 T12:V12 A10:H10 A5 C5:H5 A4:J4 O5 M5 A6:H6 M6 A7:H7 O7 M7 A8:H8 M8 A9:H9 M9 O9 M10 M11 O11 M12 A13:H13 M13 A14:H14 M14 O14 A19:H19 A18:H18 M18 O18 M19 M20 M21 M22 A23:H23 M23 O23 A24:H24 M24 O24 M25 O25 M26 M27 O27 A28:H28 M28 A29:H29 M29 A30:C30 M30 O30 J25 J23 J22 J21 J20 J19 J14 J13 J12 J10 J8 J5 A15:J17 A33:H33 A3:J3 A1:J2 E30:H30 A31:H31 J31 M31 O31 A32:C32 J32 O32 E32:H32 J33" numberStoredAsText="1"/>
   </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -4294,134 +4465,134 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B1" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="E1" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="F1" t="s">
         <v>1</v>
       </c>
       <c r="G1" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D2" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="E2" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="G2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="D3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="E3" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="G3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B4" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="D4" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E4" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="G4" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B5" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="D5" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="E5" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="B6" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="D6" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="E6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D7" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="E7" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="D8" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="E8" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="D9" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="E9" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -4466,42 +4637,42 @@
         <v>10</v>
       </c>
       <c r="I1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B2" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="G2" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="H2">
         <v>500000</v>
@@ -4510,39 +4681,39 @@
         <v>6000</v>
       </c>
       <c r="J2" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="K2" t="s">
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="M2" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="C3" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="D3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G3" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="H3" t="s">
         <v>1</v>
@@ -4551,7 +4722,7 @@
         <v>3600</v>
       </c>
       <c r="J3" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="K3" t="s">
         <v>1</v>
@@ -4560,7 +4731,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ux: admin sees focused nav (Platform + Management) only
Admin no longer sees the full FA workspace (Clients, Insurance, Investment,
Cash Flow, Meetings, Tasks, Email Hub, Templates, etc.). Admin nav:
  Platform: Dashboard, Admin Dashboard
  Management: Settings, Knowledge Base

Advisor nav is unchanged — full workspace as before.
</commit_message>
<xml_diff>
--- a/notion-import-templates/Insurance_Policies_Template.xlsx
+++ b/notion-import-templates/Insurance_Policies_Template.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="597" documentId="11_4902661BDEE849986904A2AD6474A91100A393FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{629F0596-6CED-488A-BDE5-EB11293112EC}"/>
+  <xr:revisionPtr revIDLastSave="599" documentId="11_4902661BDEE849986904A2AD6474A91100A393FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A246302-8312-495C-8719-26909F434E5D}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="225">
   <si>
     <t>Bill Morrisons — Insurance Policies Data Entry</t>
   </si>
@@ -74,12 +74,6 @@
     <t>CI Cover (MYR)</t>
   </si>
   <si>
-    <t>Early CI Cover (MYR)</t>
-  </si>
-  <si>
-    <t>Lady Cover</t>
-  </si>
-  <si>
     <t>PA Cover (MYR)</t>
   </si>
   <si>
@@ -138,12 +132,6 @@
   </si>
   <si>
     <t>Critical illness cover MYR (0 if same as SA)</t>
-  </si>
-  <si>
-    <t>Easrly CI cover MYR (0 if same as SA)</t>
-  </si>
-  <si>
-    <t>Lady cover MYR (0 if same as SA)</t>
   </si>
   <si>
     <t>Personal accident cover MYR (0 if same as SA)</t>
@@ -318,9 +306,6 @@
     <t>DORIS CHIEW JING TZE</t>
   </si>
   <si>
-    <t>🛡️ Life Cover, ⏸️ Waiver of Premium, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
-  </si>
-  <si>
     <t>0106809071</t>
   </si>
   <si>
@@ -336,16 +321,10 @@
     <t>CHAR CHEE LIM</t>
   </si>
   <si>
-    <t>🛡️ Life Cover, ♿ TPD, 🌟 Early CI</t>
-  </si>
-  <si>
     <t>0106973912</t>
   </si>
   <si>
     <t>🛡️ Life Cover, ♿ TPD, 🏥 Medical, ⏸️ Waiver of Premium</t>
-  </si>
-  <si>
-    <t>🛡️ Life Cover, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
   </si>
   <si>
     <t>0104649955</t>
@@ -717,6 +696,27 @@
   </si>
   <si>
     <t>Medical card — Panel A</t>
+  </si>
+  <si>
+    <t>Early CI Cover (MYR)</t>
+  </si>
+  <si>
+    <t>Easrly CI cover MYR (0 if same as SA)</t>
+  </si>
+  <si>
+    <t>🛡️ Life Cover, ⏸️ Waiver of Premium, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
+  </si>
+  <si>
+    <t>🛡️ Life Cover, ♿ TPD, 🌟 Early CI</t>
+  </si>
+  <si>
+    <t>🛡️ Life Cover, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
+  </si>
+  <si>
+    <t>Lady Cover</t>
+  </si>
+  <si>
+    <t>Lady cover MYR (0 if same as SA)</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -817,6 +817,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1154,7 +1158,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V61"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="27.25" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" bestFit="1" customWidth="1"/>
@@ -1178,7 +1182,7 @@
     <col min="22" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1240,7 +1244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:22">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1302,7 +1306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="16.5">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1334,137 +1338,137 @@
         <v>12</v>
       </c>
       <c r="K3" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="M3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="P3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="Q3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="R3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="S3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="T3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="1" t="s">
+      <c r="U3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="T3" s="1" t="s">
+      <c r="V3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="U3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:22" ht="47.25" x14ac:dyDescent="0.5">
+      <c r="A4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="V3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" ht="32.25">
-      <c r="A4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="F4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="G4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="H4" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="I4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="J4" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="K4" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="M4" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="N4" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="O4" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="P4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="Q4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="N4" s="8" t="s">
+      <c r="R4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="O4" s="8" t="s">
+      <c r="S4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="P4" s="6" t="s">
+      <c r="T4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="U4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="V4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="S4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="T4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="U4" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="V4" s="1" t="s">
+      <c r="C5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="5" spans="1:22">
-      <c r="A5" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="H5" s="1">
         <v>1000000</v>
       </c>
-      <c r="I5" s="6">
-        <v>0</v>
+      <c r="I5" s="1">
+        <v>1000000</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>1</v>
@@ -1473,7 +1477,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>1000000</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>1</v>
@@ -1494,30 +1498,30 @@
         <v>1</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G6" s="2">
         <v>6000739155</v>
@@ -1525,8 +1529,8 @@
       <c r="H6" s="1">
         <v>100000</v>
       </c>
-      <c r="I6" s="6">
-        <v>0</v>
+      <c r="I6" s="1">
+        <v>100000</v>
       </c>
       <c r="J6" s="1">
         <v>0</v>
@@ -1535,7 +1539,7 @@
         <v>1</v>
       </c>
       <c r="N6" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O6" s="1">
         <v>200</v>
@@ -1556,39 +1560,39 @@
         <v>1</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="V6" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:22">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="E7" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H7" s="1">
         <v>150000</v>
       </c>
-      <c r="I7" s="6">
-        <v>0</v>
+      <c r="I7" s="1">
+        <v>150000</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
@@ -1597,7 +1601,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="1">
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>1</v>
@@ -1618,39 +1622,39 @@
         <v>1</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V7" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H8" s="1">
         <v>10000</v>
       </c>
-      <c r="I8" s="6">
-        <v>0</v>
+      <c r="I8" s="1">
+        <v>10000</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>1</v>
@@ -1659,7 +1663,7 @@
         <v>1</v>
       </c>
       <c r="N8" s="1">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="O8" s="1">
         <v>150</v>
@@ -1680,39 +1684,39 @@
         <v>1</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="V8" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="H9" s="1">
         <v>50000</v>
       </c>
-      <c r="I9" s="6">
-        <v>0</v>
+      <c r="I9" s="1">
+        <v>50000</v>
       </c>
       <c r="J9" s="1">
         <v>150000</v>
@@ -1721,7 +1725,7 @@
         <v>1</v>
       </c>
       <c r="N9" s="1">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>1</v>
@@ -1742,30 +1746,30 @@
         <v>1</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="V9" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:22">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="C10" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G10" s="2">
         <v>8009558744</v>
@@ -1773,8 +1777,8 @@
       <c r="H10" s="1">
         <v>5000</v>
       </c>
-      <c r="I10" s="6">
-        <v>0</v>
+      <c r="I10" s="1">
+        <v>5000</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>1</v>
@@ -1783,7 +1787,7 @@
         <v>1</v>
       </c>
       <c r="N10" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O10" s="1">
         <v>300</v>
@@ -1804,30 +1808,30 @@
         <v>1</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V10" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G11" s="2">
         <v>8001890884</v>
@@ -1835,8 +1839,8 @@
       <c r="H11" s="1">
         <v>100000</v>
       </c>
-      <c r="I11" s="6">
-        <v>0</v>
+      <c r="I11" s="1">
+        <v>100000</v>
       </c>
       <c r="J11" s="1">
         <v>0</v>
@@ -1845,7 +1849,7 @@
         <v>1</v>
       </c>
       <c r="N11" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>1</v>
@@ -1860,36 +1864,36 @@
         <v>79103</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="T11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V11" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:22">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G12" s="2">
         <v>8010673726</v>
@@ -1897,8 +1901,8 @@
       <c r="H12" s="1">
         <v>5000</v>
       </c>
-      <c r="I12" s="6">
-        <v>0</v>
+      <c r="I12" s="1">
+        <v>5000</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>1</v>
@@ -1907,7 +1911,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O12" s="1">
         <v>200</v>
@@ -1922,36 +1926,36 @@
         <v>71660</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="T12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V12" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:22">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G13" s="2">
         <v>8010673637</v>
@@ -1959,8 +1963,8 @@
       <c r="H13" s="1">
         <v>5000</v>
       </c>
-      <c r="I13" s="6">
-        <v>0</v>
+      <c r="I13" s="1">
+        <v>5000</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>1</v>
@@ -1969,7 +1973,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O13" s="1">
         <v>200</v>
@@ -1990,30 +1994,30 @@
         <v>1</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="V13" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:22">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G14" s="2">
         <v>6001000871</v>
@@ -2021,8 +2025,8 @@
       <c r="H14" s="1">
         <v>200000</v>
       </c>
-      <c r="I14" s="6">
-        <v>0</v>
+      <c r="I14" s="1">
+        <v>200000</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>1</v>
@@ -2031,7 +2035,7 @@
         <v>1</v>
       </c>
       <c r="N14" s="1">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>1</v>
@@ -2052,30 +2056,30 @@
         <v>1</v>
       </c>
       <c r="U14" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="V14" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A15" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="V14" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22">
-      <c r="A15" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="G15" s="2">
         <v>35438762</v>
@@ -2083,8 +2087,8 @@
       <c r="H15" s="1">
         <v>1000000</v>
       </c>
-      <c r="I15" s="6" t="s">
-        <v>1</v>
+      <c r="I15" s="1">
+        <v>1000000</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>1</v>
@@ -2092,8 +2096,8 @@
       <c r="M15" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N15" s="1" t="s">
-        <v>1</v>
+      <c r="N15" s="1">
+        <v>1000000</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>1</v>
@@ -2114,30 +2118,30 @@
         <v>1</v>
       </c>
       <c r="U15" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="V15" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:22">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G16" s="2">
         <v>31359163</v>
@@ -2145,8 +2149,8 @@
       <c r="H16" s="1">
         <v>100000</v>
       </c>
-      <c r="I16" s="6" t="s">
-        <v>1</v>
+      <c r="I16" s="1">
+        <v>100000</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>1</v>
@@ -2154,8 +2158,8 @@
       <c r="M16" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N16" s="1" t="s">
-        <v>1</v>
+      <c r="N16" s="1">
+        <v>100000</v>
       </c>
       <c r="O16" s="1" t="s">
         <v>1</v>
@@ -2176,30 +2180,30 @@
         <v>1</v>
       </c>
       <c r="U16" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V16" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:22">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="G17" s="2">
         <v>35439348</v>
@@ -2207,8 +2211,8 @@
       <c r="H17" s="1">
         <v>1000000</v>
       </c>
-      <c r="I17" s="6" t="s">
-        <v>1</v>
+      <c r="I17" s="1">
+        <v>1000000</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>1</v>
@@ -2216,8 +2220,8 @@
       <c r="M17" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N17" s="1" t="s">
-        <v>1</v>
+      <c r="N17" s="1">
+        <v>1000000</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>1</v>
@@ -2238,30 +2242,30 @@
         <v>1</v>
       </c>
       <c r="U17" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="V17" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:22">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G18" s="2">
         <v>6000739226</v>
@@ -2269,8 +2273,8 @@
       <c r="H18" s="1">
         <v>100000</v>
       </c>
-      <c r="I18" s="6">
-        <v>0</v>
+      <c r="I18" s="1">
+        <v>100000</v>
       </c>
       <c r="J18" s="1">
         <v>150000</v>
@@ -2279,7 +2283,7 @@
         <v>1</v>
       </c>
       <c r="N18" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>1</v>
@@ -2300,30 +2304,30 @@
         <v>1</v>
       </c>
       <c r="U18" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="V18" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:22">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G19" s="2">
         <v>8010673612</v>
@@ -2331,8 +2335,8 @@
       <c r="H19" s="1">
         <v>5000</v>
       </c>
-      <c r="I19" s="6">
-        <v>0</v>
+      <c r="I19" s="1">
+        <v>5000</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>1</v>
@@ -2341,7 +2345,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O19" s="1">
         <v>200</v>
@@ -2362,30 +2366,30 @@
         <v>1</v>
       </c>
       <c r="U19" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="V19" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:22">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G20" s="2">
         <v>8010751037</v>
@@ -2393,8 +2397,8 @@
       <c r="H20" s="1">
         <v>5000</v>
       </c>
-      <c r="I20" s="6">
-        <v>0</v>
+      <c r="I20" s="1">
+        <v>5000</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>1</v>
@@ -2403,7 +2407,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O20" s="1">
         <v>200</v>
@@ -2418,36 +2422,36 @@
         <v>69850</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="T20" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U20" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V20" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:22">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G21" s="2">
         <v>8010750874</v>
@@ -2455,8 +2459,8 @@
       <c r="H21" s="1">
         <v>5000</v>
       </c>
-      <c r="I21" s="6">
-        <v>0</v>
+      <c r="I21" s="1">
+        <v>5000</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>1</v>
@@ -2465,7 +2469,7 @@
         <v>1</v>
       </c>
       <c r="N21" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O21" s="1">
         <v>200</v>
@@ -2483,30 +2487,30 @@
         <v>1</v>
       </c>
       <c r="U21" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="V21" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:22">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G22" s="2">
         <v>8010750804</v>
@@ -2514,8 +2518,8 @@
       <c r="H22" s="1">
         <v>5000</v>
       </c>
-      <c r="I22" s="6">
-        <v>0</v>
+      <c r="I22" s="1">
+        <v>5000</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>1</v>
@@ -2524,7 +2528,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O22" s="1">
         <v>200</v>
@@ -2539,36 +2543,36 @@
         <v>68389</v>
       </c>
       <c r="S22" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="T22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="V22" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A23" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="T22" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U22" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="V22" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:22">
-      <c r="A23" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="E23" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G23" s="2">
         <v>8003557527</v>
@@ -2576,8 +2580,8 @@
       <c r="H23" s="1">
         <v>500000</v>
       </c>
-      <c r="I23" s="6">
-        <v>0</v>
+      <c r="I23" s="1">
+        <v>500000</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>1</v>
@@ -2586,7 +2590,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="1">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="O23" s="1" t="s">
         <v>1</v>
@@ -2607,30 +2611,30 @@
         <v>1</v>
       </c>
       <c r="U23" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="V23" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:22">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G24" s="2">
         <v>6001564581</v>
@@ -2638,8 +2642,8 @@
       <c r="H24" s="1">
         <v>100000</v>
       </c>
-      <c r="I24" s="6">
-        <v>0</v>
+      <c r="I24" s="1">
+        <v>100000</v>
       </c>
       <c r="J24" s="1">
         <v>0</v>
@@ -2648,7 +2652,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O24" s="1" t="s">
         <v>1</v>
@@ -2669,30 +2673,30 @@
         <v>1</v>
       </c>
       <c r="U24" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="V24" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:22">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="E25" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G25" s="2">
         <v>8003219923</v>
@@ -2700,8 +2704,8 @@
       <c r="H25" s="1">
         <v>1000000</v>
       </c>
-      <c r="I25" s="6">
-        <v>0</v>
+      <c r="I25" s="1">
+        <v>1000000</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>1</v>
@@ -2710,7 +2714,7 @@
         <v>1</v>
       </c>
       <c r="N25" s="1">
-        <v>0</v>
+        <v>1000000</v>
       </c>
       <c r="O25" s="1" t="s">
         <v>1</v>
@@ -2731,30 +2735,30 @@
         <v>1</v>
       </c>
       <c r="U25" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="V25" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:22">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G26" s="2">
         <v>8001036225</v>
@@ -2762,8 +2766,8 @@
       <c r="H26" s="1">
         <v>100000</v>
       </c>
-      <c r="I26" s="6">
-        <v>0</v>
+      <c r="I26" s="1">
+        <v>100000</v>
       </c>
       <c r="J26" s="1">
         <v>0</v>
@@ -2772,7 +2776,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O26" s="1" t="s">
         <v>1</v>
@@ -2787,36 +2791,36 @@
         <v>79152</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="T26" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U26" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V26" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:22">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G27" s="2">
         <v>8005353726</v>
@@ -2824,8 +2828,8 @@
       <c r="H27" s="1">
         <v>100000</v>
       </c>
-      <c r="I27" s="6">
-        <v>0</v>
+      <c r="I27" s="1">
+        <v>100000</v>
       </c>
       <c r="J27" s="1">
         <v>0</v>
@@ -2834,7 +2838,7 @@
         <v>1</v>
       </c>
       <c r="N27" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O27" s="1" t="s">
         <v>1</v>
@@ -2849,45 +2853,45 @@
         <v>75857</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="T27" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U27" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V27" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:22">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="H28" s="1">
         <v>100000</v>
       </c>
-      <c r="I28" s="6">
-        <v>0</v>
+      <c r="I28" s="1">
+        <v>100000</v>
       </c>
       <c r="J28" s="1">
         <v>0</v>
@@ -2896,7 +2900,7 @@
         <v>1</v>
       </c>
       <c r="N28" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O28" s="1">
         <v>200</v>
@@ -2917,39 +2921,39 @@
         <v>1</v>
       </c>
       <c r="U28" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="V28" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:22">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H29" s="1">
         <v>100000</v>
       </c>
-      <c r="I29" s="6">
-        <v>0</v>
+      <c r="I29" s="1">
+        <v>100000</v>
       </c>
       <c r="J29" s="1">
         <v>0</v>
@@ -2958,7 +2962,7 @@
         <v>1</v>
       </c>
       <c r="N29" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O29" s="1">
         <v>200</v>
@@ -2979,39 +2983,39 @@
         <v>1</v>
       </c>
       <c r="U29" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="V29" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:22">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>94</v>
+        <v>220</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H30" s="1">
         <v>300000</v>
       </c>
-      <c r="I30" s="6">
-        <v>0</v>
+      <c r="I30" s="1">
+        <v>300000</v>
       </c>
       <c r="J30" s="1">
         <v>100000</v>
@@ -3024,7 +3028,7 @@
         <v>1</v>
       </c>
       <c r="N30" s="1">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="O30" s="1" t="s">
         <v>1</v>
@@ -3045,39 +3049,39 @@
         <v>1</v>
       </c>
       <c r="U30" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="V30" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="V30" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:22">
-      <c r="A31" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="H31" s="1">
         <v>55000</v>
       </c>
-      <c r="I31" s="6">
-        <v>0</v>
+      <c r="I31" s="1">
+        <v>55000</v>
       </c>
       <c r="J31" s="1" t="s">
         <v>1</v>
@@ -3086,7 +3090,7 @@
         <v>1</v>
       </c>
       <c r="N31" s="1">
-        <v>0</v>
+        <v>55000</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>1</v>
@@ -3107,39 +3111,39 @@
         <v>1</v>
       </c>
       <c r="U31" s="1" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="V31" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:22">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>100</v>
+        <v>221</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="H32" s="1">
         <v>10000</v>
       </c>
-      <c r="I32" s="6">
-        <v>0</v>
+      <c r="I32" s="1">
+        <v>10000</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>1</v>
@@ -3148,7 +3152,7 @@
         <v>70000</v>
       </c>
       <c r="N32" s="1">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="O32" s="1" t="s">
         <v>1</v>
@@ -3169,30 +3173,30 @@
         <v>1</v>
       </c>
       <c r="U32" s="1" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="V32" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:22">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="E33" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G33" s="2">
         <v>8009545212</v>
@@ -3200,8 +3204,8 @@
       <c r="H33" s="1">
         <v>5000</v>
       </c>
-      <c r="I33" s="6">
-        <v>0</v>
+      <c r="I33" s="1">
+        <v>5000</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>1</v>
@@ -3210,7 +3214,7 @@
         <v>1</v>
       </c>
       <c r="N33" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O33" s="1">
         <v>300</v>
@@ -3231,39 +3235,39 @@
         <v>1</v>
       </c>
       <c r="U33" s="1" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="V33" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:22">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>103</v>
+        <v>222</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="H34" s="1">
         <v>200000</v>
       </c>
-      <c r="I34" s="6">
-        <v>0</v>
+      <c r="I34" s="1">
+        <v>200000</v>
       </c>
       <c r="J34" s="1">
         <v>150000</v>
@@ -3272,77 +3276,83 @@
         <v>150000</v>
       </c>
       <c r="N34" s="1">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="P34" s="1">
         <v>2520</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="U34" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="35" spans="1:22">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F35" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="G35" s="4" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="H35" s="1">
+        <v>100000</v>
+      </c>
+      <c r="I35" s="1">
+        <v>100000</v>
+      </c>
+      <c r="N35" s="1">
         <v>100000</v>
       </c>
       <c r="P35" s="1">
         <v>2760</v>
       </c>
       <c r="Q35" s="3" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="U35" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="36" spans="1:22">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G36" s="2">
         <v>8000474682</v>
@@ -3350,46 +3360,46 @@
       <c r="H36" s="1">
         <v>50000</v>
       </c>
-      <c r="I36" s="6">
-        <v>0</v>
+      <c r="I36" s="1">
+        <v>50000</v>
       </c>
       <c r="K36" s="1">
         <v>100000</v>
       </c>
       <c r="N36" s="1">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="P36" s="1">
         <v>1800</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="37" spans="1:22">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G37" s="2">
         <v>8000474701</v>
@@ -3397,49 +3407,49 @@
       <c r="H37" s="1">
         <v>50000</v>
       </c>
-      <c r="I37" s="6">
-        <v>0</v>
+      <c r="I37" s="1">
+        <v>50000</v>
       </c>
       <c r="K37" s="1">
         <v>100000</v>
       </c>
       <c r="N37" s="1">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="P37" s="1">
         <v>1800</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="S37" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="U37" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="38" spans="1:22">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A38" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G38" s="2">
         <v>8000474735</v>
@@ -3447,49 +3457,49 @@
       <c r="H38" s="1">
         <v>50000</v>
       </c>
-      <c r="I38" s="6">
-        <v>0</v>
+      <c r="I38" s="1">
+        <v>50000</v>
       </c>
       <c r="K38" s="1">
         <v>100000</v>
       </c>
       <c r="N38" s="1">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="P38" s="1">
         <v>1800</v>
       </c>
       <c r="Q38" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="R38" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="S38" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="U38" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" ht="63" x14ac:dyDescent="0.5">
+      <c r="A39" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="R38" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="S38" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="U38" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="39" spans="1:22" ht="64.5">
-      <c r="A39" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="E39" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G39" s="2">
         <v>8000319947</v>
@@ -3497,14 +3507,14 @@
       <c r="H39" s="1">
         <v>110000</v>
       </c>
-      <c r="I39" s="6">
-        <v>0</v>
+      <c r="I39" s="1">
+        <v>110000</v>
       </c>
       <c r="K39" s="1">
         <v>100000</v>
       </c>
       <c r="N39" s="1">
-        <v>0</v>
+        <v>110000</v>
       </c>
       <c r="O39" s="1">
         <v>200</v>
@@ -3513,33 +3523,33 @@
         <v>7608</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="R39" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="U39" s="6" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="40" spans="1:22">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A40" s="1" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G40" s="2">
         <v>8001136733</v>
@@ -3547,14 +3557,14 @@
       <c r="H40" s="1">
         <v>100000</v>
       </c>
-      <c r="I40" s="6">
-        <v>0</v>
+      <c r="I40" s="1">
+        <v>100000</v>
       </c>
       <c r="J40" s="1">
         <v>0</v>
       </c>
       <c r="N40" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O40" s="1">
         <v>200</v>
@@ -3563,33 +3573,33 @@
         <v>2892</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="S40" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:22">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A41" s="1" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G41" s="2">
         <v>6000914783</v>
@@ -3597,43 +3607,43 @@
       <c r="H41" s="1">
         <v>414000</v>
       </c>
-      <c r="I41" s="6">
-        <v>0</v>
+      <c r="I41" s="1">
+        <v>414000</v>
       </c>
       <c r="N41" s="1">
-        <v>0</v>
+        <v>414000</v>
       </c>
       <c r="P41" s="1">
         <v>2400</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="U41" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="42" spans="1:22">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A42" s="1" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G42" s="2">
         <v>8009554653</v>
@@ -3641,11 +3651,11 @@
       <c r="H42" s="1">
         <v>5000</v>
       </c>
-      <c r="I42" s="6">
-        <v>0</v>
+      <c r="I42" s="1">
+        <v>5000</v>
       </c>
       <c r="N42" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O42" s="1">
         <v>300</v>
@@ -3660,27 +3670,27 @@
         <v>68427</v>
       </c>
       <c r="S42" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="43" spans="1:22" ht="16.5">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A43" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G43" s="2">
         <v>8006861955</v>
@@ -3688,11 +3698,11 @@
       <c r="H43" s="1">
         <v>500000</v>
       </c>
-      <c r="I43" s="6">
-        <v>0</v>
+      <c r="I43" s="1">
+        <v>500000</v>
       </c>
       <c r="N43" s="1">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="P43" s="1">
         <v>2499.96</v>
@@ -3704,42 +3714,42 @@
         <v>61271</v>
       </c>
       <c r="U43" s="6" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="44" spans="1:22" ht="48.75">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" ht="47.25" x14ac:dyDescent="0.5">
       <c r="A44" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="H44" s="1">
         <v>100000</v>
       </c>
-      <c r="I44" s="6">
-        <v>0</v>
+      <c r="I44" s="1">
+        <v>100000</v>
       </c>
       <c r="J44" s="1">
         <v>0</v>
       </c>
       <c r="N44" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="P44" s="1">
         <v>1800</v>
@@ -3751,74 +3761,74 @@
         <v>68181</v>
       </c>
       <c r="U44" s="6" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="45" spans="1:22" ht="32.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A45" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B45" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C45" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="E45" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H45" s="1">
         <v>160000</v>
       </c>
-      <c r="I45" s="6">
-        <v>0</v>
+      <c r="I45" s="1">
+        <v>160000</v>
       </c>
       <c r="J45" s="1">
         <v>0</v>
       </c>
       <c r="N45" s="1">
-        <v>0</v>
+        <v>160000</v>
       </c>
       <c r="P45" s="1">
         <v>1200</v>
       </c>
       <c r="Q45" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="R45" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="U45" s="6" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="46" spans="1:22">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A46" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G46" s="2">
         <v>8010004645</v>
@@ -3826,11 +3836,11 @@
       <c r="H46" s="1">
         <v>5000</v>
       </c>
-      <c r="I46" s="6">
-        <v>0</v>
+      <c r="I46" s="1">
+        <v>5000</v>
       </c>
       <c r="N46" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O46" s="1">
         <v>200</v>
@@ -3845,34 +3855,40 @@
         <v>57202</v>
       </c>
       <c r="U46" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A47" s="1" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="47" spans="1:22">
-      <c r="A47" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="B47" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C47" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="G47" s="4" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H47" s="1">
         <v>1000000</v>
       </c>
+      <c r="I47" s="1">
+        <v>1000000</v>
+      </c>
+      <c r="N47" s="1">
+        <v>1000000</v>
+      </c>
       <c r="P47" s="1">
         <v>5340</v>
       </c>
@@ -3883,36 +3899,36 @@
         <v>68215</v>
       </c>
       <c r="U47" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="48" spans="1:22">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A48" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="H48" s="1">
         <v>100000</v>
       </c>
-      <c r="I48" s="6">
-        <v>0</v>
+      <c r="I48" s="1">
+        <v>100000</v>
       </c>
       <c r="J48" s="1">
         <v>0</v>
@@ -3921,7 +3937,7 @@
         <v>50000</v>
       </c>
       <c r="N48" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O48" s="1">
         <v>200</v>
@@ -3936,27 +3952,27 @@
         <v>68368</v>
       </c>
       <c r="U48" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="49" spans="1:21" ht="32.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="49" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A49" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G49" s="2">
         <v>6001549235</v>
@@ -3964,119 +3980,131 @@
       <c r="H49" s="1">
         <v>600000</v>
       </c>
-      <c r="I49" s="6">
-        <v>0</v>
+      <c r="I49" s="1">
+        <v>600000</v>
       </c>
       <c r="N49" s="1">
-        <v>0</v>
+        <v>600000</v>
       </c>
       <c r="P49" s="1">
         <v>1440</v>
       </c>
       <c r="Q49" s="3" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="R49" s="3" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="U49" s="6" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="50" spans="1:21" ht="32.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A50" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G50" s="4" t="s">
         <v>142</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>149</v>
       </c>
       <c r="H50" s="1">
         <v>50000</v>
       </c>
+      <c r="I50" s="1">
+        <v>50000</v>
+      </c>
+      <c r="N50" s="1">
+        <v>50000</v>
+      </c>
       <c r="P50" s="1">
         <v>1500</v>
       </c>
       <c r="Q50" s="3" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="R50" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="U50" s="6" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="51" spans="1:21">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A51" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="H51" s="1">
         <v>150000</v>
       </c>
+      <c r="I51" s="1">
+        <v>150000</v>
+      </c>
+      <c r="N51" s="1">
+        <v>150000</v>
+      </c>
       <c r="P51" s="1">
         <v>1200</v>
       </c>
       <c r="Q51" s="3" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="R51" s="3" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="U51" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="52" spans="1:21" ht="32.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="52" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A52" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G52" s="2">
         <v>8005001007</v>
@@ -4084,6 +4112,12 @@
       <c r="H52" s="1">
         <v>600000</v>
       </c>
+      <c r="I52" s="1">
+        <v>600000</v>
+      </c>
+      <c r="N52" s="1">
+        <v>600000</v>
+      </c>
       <c r="P52" s="1">
         <v>2400</v>
       </c>
@@ -4094,27 +4128,27 @@
         <v>61214</v>
       </c>
       <c r="U52" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.5">
+      <c r="A53" s="1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="53" spans="1:21">
-      <c r="A53" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="B53" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G53" s="2">
         <v>8009518746</v>
@@ -4122,37 +4156,43 @@
       <c r="H53" s="1">
         <v>5000</v>
       </c>
+      <c r="I53" s="1">
+        <v>5000</v>
+      </c>
+      <c r="N53" s="1">
+        <v>5000</v>
+      </c>
       <c r="P53" s="1">
         <v>3132</v>
       </c>
       <c r="Q53" s="3" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="R53" s="3" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="U53" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="54" spans="1:21">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A54" s="1" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G54" s="2">
         <v>8005001052</v>
@@ -4160,6 +4200,12 @@
       <c r="H54" s="1">
         <v>1500000</v>
       </c>
+      <c r="I54" s="1">
+        <v>1500000</v>
+      </c>
+      <c r="N54" s="1">
+        <v>1500000</v>
+      </c>
       <c r="P54" s="1">
         <v>6000</v>
       </c>
@@ -4170,27 +4216,27 @@
         <v>56984</v>
       </c>
       <c r="U54" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="55" spans="1:21" ht="16.5">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A55" s="1" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G55" s="2">
         <v>6001512162</v>
@@ -4198,37 +4244,43 @@
       <c r="H55" s="1">
         <v>100000</v>
       </c>
+      <c r="I55" s="1">
+        <v>100000</v>
+      </c>
+      <c r="N55" s="1">
+        <v>100000</v>
+      </c>
       <c r="P55" s="1">
         <v>1800</v>
       </c>
       <c r="Q55" s="3" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="R55" s="3" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="U55" s="6" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="56" spans="1:21">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A56" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G56" s="2">
         <v>8002084775</v>
@@ -4236,46 +4288,52 @@
       <c r="H56" s="1">
         <v>100000</v>
       </c>
+      <c r="I56" s="1">
+        <v>100000</v>
+      </c>
+      <c r="N56" s="1">
+        <v>100000</v>
+      </c>
       <c r="P56" s="1">
         <v>12000</v>
       </c>
       <c r="Q56" s="3" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="R56" s="3" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="U56" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="57" spans="1:21">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="57" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A57" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C57" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="G57" s="4" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="H57" s="1">
         <v>100000</v>
       </c>
-      <c r="I57" s="6">
-        <v>0</v>
+      <c r="I57" s="1">
+        <v>100000</v>
       </c>
       <c r="J57" s="9">
         <v>200000</v>
@@ -4283,41 +4341,47 @@
       <c r="K57" s="9"/>
       <c r="L57" s="9"/>
       <c r="N57" s="1">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="P57" s="1">
         <v>2400</v>
       </c>
       <c r="Q57" s="3" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="R57" s="3" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="58" spans="1:21" ht="32.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="58" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A58" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H58" s="1">
+        <v>100000</v>
+      </c>
+      <c r="I58" s="1">
+        <v>100000</v>
+      </c>
+      <c r="N58" s="1">
         <v>100000</v>
       </c>
       <c r="P58" s="1">
@@ -4330,34 +4394,40 @@
         <v>68282</v>
       </c>
       <c r="U58" s="6" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="59" spans="1:21" ht="32.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A59" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G59" s="4" t="s">
         <v>167</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G59" s="4" t="s">
-        <v>174</v>
       </c>
       <c r="H59" s="1">
         <v>150000</v>
       </c>
+      <c r="I59" s="1">
+        <v>150000</v>
+      </c>
+      <c r="N59" s="1">
+        <v>150000</v>
+      </c>
       <c r="P59" s="1">
         <v>3000</v>
       </c>
@@ -4368,27 +4438,27 @@
         <v>68184</v>
       </c>
       <c r="U59" s="6" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="60" spans="1:21">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="60" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A60" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G60" s="2">
         <v>8010660964</v>
@@ -4396,6 +4466,12 @@
       <c r="H60" s="1">
         <v>5000</v>
       </c>
+      <c r="I60" s="1">
+        <v>5000</v>
+      </c>
+      <c r="N60" s="1">
+        <v>5000</v>
+      </c>
       <c r="P60" s="1">
         <v>3672</v>
       </c>
@@ -4406,32 +4482,38 @@
         <v>61064</v>
       </c>
       <c r="U60" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="61" spans="1:21">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="61" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A61" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="H61" s="1">
+        <v>500000</v>
+      </c>
+      <c r="I61" s="1">
+        <v>500000</v>
+      </c>
+      <c r="N61" s="1">
         <v>500000</v>
       </c>
       <c r="P61" s="1">
@@ -4447,7 +4529,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="M1:V2 M3:O3 S3:V10 M33 B26:H26 O26 A25:H25 B22:H22 S23:V25 T20:V20 A21:H21 B20:H20 T21:V21 T22:V22 S28:V33 T26:V26 B27:H27 T27:V27 S13:V19 T11:V11 M15:O17 B11:H11 B12:H12 T12:V12 A10:H10 A5 C5:H5 A4:J4 O5 M5 A6:H6 M6 A7:H7 O7 M7 A8:H8 M8 A9:H9 M9 O9 M10 M11 O11 M12 A13:H13 M13 A14:H14 M14 O14 A19:H19 A18:H18 M18 O18 M19 M20 M21 M22 A23:H23 M23 O23 A24:H24 M24 O24 M25 O25 M26 M27 O27 A28:H28 M28 A29:H29 M29 A30:C30 M30 O30 J25 J23 J22 J21 J20 J19 J14 J13 J12 J10 J8 J5 A15:J17 A33:H33 A3:J3 A1:J2 E30:H30 A31:H31 J31 M31 O31 A32:C32 J32 O32 E32:H32 J33" numberStoredAsText="1"/>
+    <ignoredError sqref="M1:V2 M3:O4 S3:V10 M33 B22:H22 S23:V25 A21:H21 B20:H20 T20:V22 S28:V33 B26:H27 T26:V27 S13:V19 M15:M17 B11:H12 T11:V12 A5 C5:H5 O5 O7 A6:H10 O9 O11 A13:H14 M5:M14 O14 A18:H19 O18 A23:H25 O23:O27 A28:H29 M18:M30 O30 J25 J19:J23 J12:J14 J10 J8 A15:H17 A33:H33 A1:J4 A30:C30 E30:H30 A31:H31 J31 M31 O31 A32:C32 J32 O32 E32:H32 J33 J15:J17 O15:O17" numberStoredAsText="1"/>
   </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -4458,141 +4540,141 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="4" max="4" width="27.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>175</v>
+      </c>
+      <c r="E1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
+        <v>178</v>
+      </c>
+      <c r="D2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E2" t="s">
         <v>180</v>
       </c>
-      <c r="B1" t="s">
+      <c r="G2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A3" t="s">
         <v>181</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="B3" t="s">
         <v>182</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D3" t="s">
         <v>183</v>
       </c>
-      <c r="F1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="E3" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="G3" t="s">
         <v>185</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A4" t="s">
         <v>186</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B4" t="s">
         <v>187</v>
       </c>
-      <c r="G2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
+      <c r="D4" t="s">
         <v>188</v>
       </c>
-      <c r="B3" t="s">
+      <c r="E4" t="s">
         <v>189</v>
       </c>
-      <c r="D3" t="s">
+      <c r="G4" t="s">
         <v>190</v>
       </c>
-      <c r="E3" t="s">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A5" t="s">
         <v>191</v>
       </c>
-      <c r="G3" t="s">
+      <c r="B5" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
+      <c r="D5" t="s">
         <v>193</v>
       </c>
-      <c r="B4" t="s">
+      <c r="E5" t="s">
         <v>194</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A6" t="s">
         <v>195</v>
       </c>
-      <c r="E4" t="s">
+      <c r="B6" t="s">
         <v>196</v>
       </c>
-      <c r="G4" t="s">
+      <c r="D6" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
+      <c r="E6" t="s">
         <v>198</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" t="s">
         <v>199</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D7" t="s">
         <v>200</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="D8" t="s">
         <v>202</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E8" t="s">
         <v>203</v>
       </c>
-      <c r="D6" t="s">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="D9" t="s">
         <v>204</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E9" t="s">
         <v>205</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" t="s">
-        <v>206</v>
-      </c>
-      <c r="D7" t="s">
-        <v>207</v>
-      </c>
-      <c r="E7" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="D8" t="s">
-        <v>209</v>
-      </c>
-      <c r="E8" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="D9" t="s">
-        <v>211</v>
-      </c>
-      <c r="E9" t="s">
-        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -4606,12 +4688,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="12" max="12" width="13.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -4637,42 +4719,42 @@
         <v>10</v>
       </c>
       <c r="I1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" t="s">
         <v>18</v>
       </c>
-      <c r="J1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K1" t="s">
-        <v>20</v>
-      </c>
       <c r="L1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B2" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D2" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="G2" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="H2">
         <v>500000</v>
@@ -4681,39 +4763,39 @@
         <v>6000</v>
       </c>
       <c r="J2" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="K2" t="s">
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="M2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B3" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="C3" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="D3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G3" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="H3" t="s">
         <v>1</v>
@@ -4722,7 +4804,7 @@
         <v>3600</v>
       </c>
       <c r="J3" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="K3" t="s">
         <v>1</v>
@@ -4731,7 +4813,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: insurance template clarity + Medical Card details
- Rename template column 'Client Name *' → 'Policy Owner *' so the linked
  client is clearly the policy owner (assistants were putting Life Assured in
  the old ambiguous 'Client Name')
- Repurpose the duplicate 'Policy Owner' column → 'Medical Card (R&B / Annual
  Limit)' for medical card details in one column
- Import script reads Policy Owner * (fallback Client Name *) for the client
  link + Policy Owner field; imports Medical Card; Life Assured unchanged
- Notion Insurance DB: added 'Medical Card' property
- Insurance API + page: surface Medical Card next to Medical Class

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/Insurance_Policies_Template.xlsx
+++ b/notion-import-templates/Insurance_Policies_Template.xlsx
@@ -1,39 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="599" documentId="11_4902661BDEE849986904A2AD6474A91100A393FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A246302-8312-495C-8719-26909F434E5D}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155"/>
   </bookViews>
   <sheets>
-    <sheet name="Insurance Policies" sheetId="1" r:id="rId1"/>
-    <sheet name="Reference" sheetId="2" r:id="rId2"/>
-    <sheet name="Sample" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Insurance Policies" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Reference" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Sample" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="227">
   <si>
     <t>Bill Morrisons — Insurance Policies Data Entry</t>
   </si>
@@ -44,7 +27,7 @@
     <t>Template generated 20/05/2026 · Fill in all yellow columns · Dates format: DD/MM/YYYY · Benefits: separate multiple with comma</t>
   </si>
   <si>
-    <t>Client Name *</t>
+    <t>Policy Owner *</t>
   </si>
   <si>
     <t>Policy Name *</t>
@@ -74,6 +57,12 @@
     <t>CI Cover (MYR)</t>
   </si>
   <si>
+    <t>Early CI Cover (MYR)</t>
+  </si>
+  <si>
+    <t>Lady Cover</t>
+  </si>
+  <si>
     <t>PA Cover (MYR)</t>
   </si>
   <si>
@@ -92,7 +81,7 @@
     <t>Maturity Date</t>
   </si>
   <si>
-    <t>Policy Owner</t>
+    <t>Medical Card (R&amp;B / Annual Limit)</t>
   </si>
   <si>
     <t>Life Assured</t>
@@ -104,7 +93,7 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Must match Clients DB</t>
+    <t>Policy owner — must match a name in your Clients database</t>
   </si>
   <si>
     <t>Full policy name</t>
@@ -134,6 +123,12 @@
     <t>Critical illness cover MYR (0 if same as SA)</t>
   </si>
   <si>
+    <t>Easrly CI cover MYR (0 if same as SA)</t>
+  </si>
+  <si>
+    <t>Lady cover MYR (0 if same as SA)</t>
+  </si>
+  <si>
     <t>Personal accident cover MYR (0 if same as SA)</t>
   </si>
   <si>
@@ -152,7 +147,7 @@
     <t>DD/MM/YYYY or blank</t>
   </si>
   <si>
-    <t>Policy owner name (blank = same as client)</t>
+    <t>e.g. R&amp;B RM250 / Annual RM2,000,000 (leave blank if no medical card)</t>
   </si>
   <si>
     <t>Life assured name (blank = same as client)</t>
@@ -185,6 +180,9 @@
     <t>00042420</t>
   </si>
   <si>
+    <t>R&amp;B RM250 / Annual RM2,000,000</t>
+  </si>
+  <si>
     <t>NIL</t>
   </si>
   <si>
@@ -233,12 +231,12 @@
     <t>AssuredLink</t>
   </si>
   <si>
+    <t>LEONG CHEE KEONG</t>
+  </si>
+  <si>
     <t>RACHEL LEONG HUI QI</t>
   </si>
   <si>
-    <t>LEONG CHEE KEONG</t>
-  </si>
-  <si>
     <t>🛡️ Life Cover, ♿ TPD, 🏥 Medical</t>
   </si>
   <si>
@@ -269,12 +267,12 @@
     <t>🛡️ Life Cover, ⏸️ Waiver of Premium</t>
   </si>
   <si>
+    <t>LOH SHI SHENG</t>
+  </si>
+  <si>
     <t>LOH LI YUAN</t>
   </si>
   <si>
-    <t>LOH SHI SHENG</t>
-  </si>
-  <si>
     <t>CHAI YOKE FOONG</t>
   </si>
   <si>
@@ -287,7 +285,7 @@
     <t>🛡️ Life Cover, ♿ TPD</t>
   </si>
   <si>
-    <t>1.LOH LI YAO_x000D_
+    <t xml:space="preserve">1.LOH LI YAO
 2. CHAI YOKE FOONG</t>
   </si>
   <si>
@@ -306,6 +304,9 @@
     <t>DORIS CHIEW JING TZE</t>
   </si>
   <si>
+    <t>🛡️ Life Cover, ⏸️ Waiver of Premium, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
+  </si>
+  <si>
     <t>0106809071</t>
   </si>
   <si>
@@ -321,12 +322,18 @@
     <t>CHAR CHEE LIM</t>
   </si>
   <si>
+    <t>🛡️ Life Cover, ♿ TPD, 🌟 Early CI</t>
+  </si>
+  <si>
     <t>0106973912</t>
   </si>
   <si>
     <t>🛡️ Life Cover, ♿ TPD, 🏥 Medical, ⏸️ Waiver of Premium</t>
   </si>
   <si>
+    <t>🛡️ Life Cover, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
+  </si>
+  <si>
     <t>0104649955</t>
   </si>
   <si>
@@ -345,33 +352,33 @@
     <t>28/01/2085</t>
   </si>
   <si>
+    <t>TAN PIEH FANG</t>
+  </si>
+  <si>
+    <t>🛡️ Life Cover, ♿ TPD,  ⏸️ Waiver of Premium, 🌟 Early CI</t>
+  </si>
+  <si>
+    <t>21/12/2016</t>
+  </si>
+  <si>
+    <t>21/12/2096</t>
+  </si>
+  <si>
     <t>CHAN JIN HAO</t>
   </si>
   <si>
-    <t>🛡️ Life Cover, ♿ TPD,  ⏸️ Waiver of Premium, 🌟 Early CI</t>
-  </si>
-  <si>
-    <t>21/12/2016</t>
-  </si>
-  <si>
-    <t>21/12/2096</t>
-  </si>
-  <si>
-    <t>TAN PIEH FANG</t>
+    <t>21/12/2098</t>
   </si>
   <si>
     <t>CHAN YUAN LIN</t>
   </si>
   <si>
-    <t>21/12/2098</t>
+    <t>21/12/2105</t>
   </si>
   <si>
     <t>CHAN SHI LING</t>
   </si>
   <si>
-    <t>21/12/2105</t>
-  </si>
-  <si>
     <t>🛡️ Life Cover, ⏸️ Waiver of Premium, 🌟 Early CI, ♿ TPD, 🏥 Medical</t>
   </si>
   <si>
@@ -381,24 +388,24 @@
     <t>22/09/2073</t>
   </si>
   <si>
-    <t>1. CHAN YUAN LIN
+    <t xml:space="preserve">1. CHAN YUAN LIN
 2. CHAN SHI LING
 3. CHAN CHEE KENG
 4. CHAN JIN HAO</t>
   </si>
   <si>
+    <t>LIM WOOI KHANG</t>
+  </si>
+  <si>
+    <t>26/10/2017</t>
+  </si>
+  <si>
+    <t>26/10/2117</t>
+  </si>
+  <si>
     <t>RAEGAN LIM SZE RAYE</t>
   </si>
   <si>
-    <t>26/10/2017</t>
-  </si>
-  <si>
-    <t>26/10/2117</t>
-  </si>
-  <si>
-    <t>LIM WOOI KHANG</t>
-  </si>
-  <si>
     <t>19/03/2015</t>
   </si>
   <si>
@@ -420,7 +427,7 @@
     <t>0102728587</t>
   </si>
   <si>
-    <t>1. LIM YEE FEI
+    <t xml:space="preserve">1. LIM YEE FEI
 2. LEONG AH LUAN
 3. LIM SHENG YEE</t>
   </si>
@@ -434,7 +441,7 @@
     <t>23/10/2086</t>
   </si>
   <si>
-    <t>1. LEONG AH LUAN
+    <t xml:space="preserve">1. LEONG AH LUAN
 2. LIM SHENG YEE</t>
   </si>
   <si>
@@ -465,7 +472,7 @@
     <t>15/07/2087</t>
   </si>
   <si>
-    <t>1. TOH HONG SHII
+    <t xml:space="preserve">1. TOH HONG SHII
 2. LIM BEE BEE</t>
   </si>
   <si>
@@ -538,7 +545,7 @@
     <t>0103101505</t>
   </si>
   <si>
-    <t>1. LEE YUK SONG
+    <t xml:space="preserve">1. LEE YUK SONG
 2. LIU KAI YOU</t>
   </si>
   <si>
@@ -662,6 +669,9 @@
     <t>Premiums waived if policy owner (parent) dies/disabled</t>
   </si>
   <si>
+    <t>Client Name *</t>
+  </si>
+  <si>
     <t>Ahmad Rizal bin Abdullah</t>
   </si>
   <si>
@@ -696,43 +706,29 @@
   </si>
   <si>
     <t>Medical card — Panel A</t>
-  </si>
-  <si>
-    <t>Early CI Cover (MYR)</t>
-  </si>
-  <si>
-    <t>Easrly CI cover MYR (0 if same as SA)</t>
-  </si>
-  <si>
-    <t>🛡️ Life Cover, ⏸️ Waiver of Premium, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
-  </si>
-  <si>
-    <t>🛡️ Life Cover, ♿ TPD, 🌟 Early CI</t>
-  </si>
-  <si>
-    <t>🛡️ Life Cover, ❤️ Critical Illness (CI), 🌟 Early CI, ♿ TPD</t>
-  </si>
-  <si>
-    <t>Lady Cover</t>
-  </si>
-  <si>
-    <t>Lady cover MYR (0 if same as SA)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -755,59 +751,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
-      <alignment horizontal="center" vertical="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
-      <alignment horizontal="center" vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-  </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -819,17 +794,17 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{69E5B004-7BF1-42CC-BE29-6E2C6D39DB56}" name="Table1" displayName="Table1" ref="P3:R33" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
-  <autoFilter ref="P3:R33" xr:uid="{69E5B004-7BF1-42CC-BE29-6E2C6D39DB56}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Table1" displayName="Table1" ref="P3:R33" totalsRowShown="1" headerRowCount="0">
+  <autoFilter ref="P3:R33">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{58D46586-83F1-4520-BB84-8DECA7EF760D}" name="Annual Premium (MYR)" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{0829D2FE-2862-4852-907C-03838995F0B3}" name="Commencement Date" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{8694827B-7786-4F19-9FDD-25C3897B6953}" name="Maturity Date" dataDxfId="0"/>
+    <tableColumn id="1" name="Annual Premium (MYR)"/>
+    <tableColumn id="2" name="Commencement Date"/>
+    <tableColumn id="3" name="Maturity Date"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1156,33 +1131,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:V61"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="27.25" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="68" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="31.625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="68" style="1" customWidth="1"/>
     <col min="5" max="5" width="21.5" style="1" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.625" style="2" customWidth="1"/>
     <col min="8" max="8" width="22.25" style="1" customWidth="1"/>
-    <col min="9" max="9" width="25.25" style="6" customWidth="1"/>
+    <col min="9" max="9" width="25.25" style="3" customWidth="1"/>
     <col min="10" max="12" width="21" style="1" customWidth="1"/>
     <col min="13" max="13" width="20.5" style="1" customWidth="1"/>
     <col min="14" max="14" width="35.75" style="1" customWidth="1"/>
     <col min="15" max="15" width="29.375" style="1" customWidth="1"/>
-    <col min="16" max="16" width="21.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.125" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="35.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9" style="1"/>
-    <col min="21" max="21" width="28.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="16384" width="9" style="1"/>
+    <col min="16" max="16" width="21.75" style="1" customWidth="1"/>
+    <col min="17" max="17" width="20.625" style="4" customWidth="1"/>
+    <col min="18" max="18" width="19.125" style="4" customWidth="1"/>
+    <col min="19" max="19" width="35.75" style="1" customWidth="1"/>
+    <col min="20" max="20" width="35.3125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="28.375" style="1" customWidth="1"/>
+    <col min="22" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1207,7 +1182,7 @@
       <c r="H1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="J1" s="1" t="s">
@@ -1225,7 +1200,7 @@
       <c r="P1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="R1" s="2" t="s">
@@ -1244,7 +1219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1269,7 +1244,7 @@
       <c r="H2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="J2" s="1" t="s">
@@ -1287,7 +1262,7 @@
       <c r="P2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Q2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="R2" s="2" t="s">
@@ -1306,7 +1281,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1319,150 +1294,150 @@
       <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="5" t="s">
         <v>11</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>218</v>
+        <v>13</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>223</v>
+        <v>14</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22" ht="47.25" x14ac:dyDescent="0.5">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" ht="31.5" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="E4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="F4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="G4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="H4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="K4" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="M4" s="8" t="s">
+      <c r="I4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N4" s="8" t="s">
+      <c r="J4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="O4" s="8" t="s">
+      <c r="K4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="P4" s="6" t="s">
+      <c r="L4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="M4" s="5" t="s">
         <v>37</v>
       </c>
+      <c r="N4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q4" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="R4" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.5">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="H5" s="1">
         <v>1000000</v>
@@ -1485,43 +1460,43 @@
       <c r="P5" s="1">
         <v>5340</v>
       </c>
-      <c r="Q5" s="3">
+      <c r="Q5" s="4">
         <v>43444</v>
       </c>
-      <c r="R5" s="3">
+      <c r="R5" s="4">
         <v>68281</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G6" s="2">
         <v>6000739155</v>
@@ -1547,46 +1522,46 @@
       <c r="P6" s="1">
         <v>3204</v>
       </c>
-      <c r="Q6" s="3">
+      <c r="Q6" s="4">
         <v>41968</v>
       </c>
-      <c r="R6" s="3">
+      <c r="R6" s="4">
         <v>68266</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="V6" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H7" s="1">
         <v>150000</v>
@@ -1609,46 +1584,46 @@
       <c r="P7" s="1">
         <v>1200</v>
       </c>
-      <c r="Q7" s="3">
+      <c r="Q7" s="4">
         <v>41291</v>
       </c>
-      <c r="R7" s="3">
+      <c r="R7" s="4">
         <v>68319</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V7" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="G8" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="H8" s="1">
         <v>10000</v>
@@ -1671,46 +1646,46 @@
       <c r="P8" s="1">
         <v>3960</v>
       </c>
-      <c r="Q8" s="3">
+      <c r="Q8" s="4">
         <v>43517</v>
       </c>
-      <c r="R8" s="3">
+      <c r="R8" s="4">
         <v>60684</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="V8" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H9" s="1">
         <v>50000</v>
@@ -1733,43 +1708,43 @@
       <c r="P9" s="1">
         <v>1800</v>
       </c>
-      <c r="Q9" s="3">
+      <c r="Q9" s="4">
         <v>42252</v>
       </c>
-      <c r="R9" s="3">
+      <c r="R9" s="4">
         <v>65263</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>1</v>
+        <v>66</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>1</v>
+        <v>66</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="V9" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="G10" s="2">
         <v>8009558744</v>
@@ -1795,43 +1770,43 @@
       <c r="P10" s="1">
         <v>4020</v>
       </c>
-      <c r="Q10" s="3">
+      <c r="Q10" s="4">
         <v>45783</v>
       </c>
-      <c r="R10" s="3">
+      <c r="R10" s="4">
         <v>54184</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>1</v>
+        <v>66</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>1</v>
+        <v>66</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V10" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G11" s="2">
         <v>8001890884</v>
@@ -1857,43 +1832,43 @@
       <c r="P11" s="1">
         <v>1800</v>
       </c>
-      <c r="Q11" s="3">
+      <c r="Q11" s="4">
         <v>43309</v>
       </c>
-      <c r="R11" s="3">
+      <c r="R11" s="4">
         <v>79103</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>1</v>
+        <v>72</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V11" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G12" s="2">
         <v>8010673726</v>
@@ -1919,43 +1894,43 @@
       <c r="P12" s="1">
         <v>1896</v>
       </c>
-      <c r="Q12" s="3">
+      <c r="Q12" s="4">
         <v>46092</v>
       </c>
-      <c r="R12" s="3">
+      <c r="R12" s="4">
         <v>71660</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>1</v>
+        <v>72</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V12" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G13" s="2">
         <v>8010673637</v>
@@ -1981,43 +1956,43 @@
       <c r="P13" s="1">
         <v>5604</v>
       </c>
-      <c r="Q13" s="3">
+      <c r="Q13" s="4">
         <v>46092</v>
       </c>
-      <c r="R13" s="3">
+      <c r="R13" s="4">
         <v>57415</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="T13" s="1" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="V13" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G14" s="2">
         <v>6001000871</v>
@@ -2043,43 +2018,43 @@
       <c r="P14" s="1">
         <v>2400</v>
       </c>
-      <c r="Q14" s="3">
+      <c r="Q14" s="4">
         <v>42142</v>
       </c>
-      <c r="R14" s="3">
+      <c r="R14" s="4">
         <v>64788</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="U14" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="V14" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="G15" s="2">
         <v>35438762</v>
@@ -2105,43 +2080,43 @@
       <c r="P15" s="1">
         <v>7392</v>
       </c>
-      <c r="Q15" s="3">
+      <c r="Q15" s="4">
         <v>43344</v>
       </c>
-      <c r="R15" s="3">
+      <c r="R15" s="4">
         <v>64529</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="T15" s="1" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="U15" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="V15" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="G16" s="2">
         <v>31359163</v>
@@ -2167,43 +2142,43 @@
       <c r="P16" s="1">
         <v>5868.6</v>
       </c>
-      <c r="Q16" s="3">
+      <c r="Q16" s="4">
         <v>45292</v>
       </c>
-      <c r="R16" s="3">
+      <c r="R16" s="4">
         <v>57346</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="T16" s="1" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="U16" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V16" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="G17" s="2">
         <v>35439348</v>
@@ -2229,43 +2204,43 @@
       <c r="P17" s="1">
         <v>6924</v>
       </c>
-      <c r="Q17" s="3">
+      <c r="Q17" s="4">
         <v>43344</v>
       </c>
-      <c r="R17" s="3">
+      <c r="R17" s="4">
         <v>66355</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="T17" s="1" t="s">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="U17" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="V17" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="V17" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.5">
-      <c r="A18" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="B18" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G18" s="2">
         <v>6000739226</v>
@@ -2291,43 +2266,43 @@
       <c r="P18" s="1">
         <v>2400</v>
       </c>
-      <c r="Q18" s="3">
+      <c r="Q18" s="4">
         <v>41969</v>
       </c>
-      <c r="R18" s="3">
+      <c r="R18" s="4">
         <v>66806</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="T18" s="1" t="s">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="U18" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="V18" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G19" s="2">
         <v>8010673612</v>
@@ -2353,43 +2328,43 @@
       <c r="P19" s="1">
         <v>4200</v>
       </c>
-      <c r="Q19" s="3">
+      <c r="Q19" s="4">
         <v>46092</v>
       </c>
-      <c r="R19" s="3">
+      <c r="R19" s="4">
         <v>59241</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="U19" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="V19" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G20" s="2">
         <v>8010751037</v>
@@ -2415,43 +2390,43 @@
       <c r="P20" s="1">
         <v>1824</v>
       </c>
-      <c r="Q20" s="3">
+      <c r="Q20" s="4">
         <v>46111</v>
       </c>
-      <c r="R20" s="3">
+      <c r="R20" s="4">
         <v>69850</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="U20" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V20" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G21" s="2">
         <v>8010750874</v>
@@ -2477,40 +2452,43 @@
       <c r="P21" s="1">
         <v>4248</v>
       </c>
-      <c r="Q21" s="3">
+      <c r="Q21" s="4">
         <v>46111</v>
       </c>
-      <c r="R21" s="3">
+      <c r="R21" s="4">
         <v>60719</v>
       </c>
+      <c r="S21" s="1" t="s">
+        <v>83</v>
+      </c>
       <c r="T21" s="1" t="s">
-        <v>1</v>
+        <v>83</v>
       </c>
       <c r="U21" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="V21" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G22" s="2">
         <v>8010750804</v>
@@ -2536,43 +2514,43 @@
       <c r="P22" s="1">
         <v>1848</v>
       </c>
-      <c r="Q22" s="3">
+      <c r="Q22" s="4">
         <v>46111</v>
       </c>
-      <c r="R22" s="3">
+      <c r="R22" s="4">
         <v>68389</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="T22" s="1" t="s">
-        <v>1</v>
+        <v>86</v>
       </c>
       <c r="U22" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V22" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G23" s="2">
         <v>8003557527</v>
@@ -2598,43 +2576,43 @@
       <c r="P23" s="1">
         <v>1800</v>
       </c>
-      <c r="Q23" s="3">
+      <c r="Q23" s="4">
         <v>43859</v>
       </c>
-      <c r="R23" s="3">
+      <c r="R23" s="4">
         <v>54816</v>
       </c>
       <c r="S23" s="1" t="s">
-        <v>1</v>
+        <v>83</v>
       </c>
       <c r="T23" s="1" t="s">
-        <v>1</v>
+        <v>83</v>
       </c>
       <c r="U23" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="V23" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G24" s="2">
         <v>6001564581</v>
@@ -2660,43 +2638,43 @@
       <c r="P24" s="1">
         <v>1800</v>
       </c>
-      <c r="Q24" s="3">
+      <c r="Q24" s="4">
         <v>42621</v>
       </c>
-      <c r="R24" s="3">
+      <c r="R24" s="4">
         <v>68188</v>
       </c>
       <c r="S24" s="1" t="s">
-        <v>1</v>
+        <v>83</v>
       </c>
       <c r="T24" s="1" t="s">
-        <v>1</v>
+        <v>83</v>
       </c>
       <c r="U24" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="V24" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G25" s="2">
         <v>8003219923</v>
@@ -2722,43 +2700,43 @@
       <c r="P25" s="1">
         <v>2232</v>
       </c>
-      <c r="Q25" s="3">
+      <c r="Q25" s="4">
         <v>43752</v>
       </c>
-      <c r="R25" s="3">
+      <c r="R25" s="4">
         <v>51423</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>1</v>
+        <v>83</v>
       </c>
       <c r="T25" s="1" t="s">
-        <v>1</v>
+        <v>83</v>
       </c>
       <c r="U25" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="V25" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G26" s="2">
         <v>8001036225</v>
@@ -2784,43 +2762,43 @@
       <c r="P26" s="1">
         <v>1200</v>
       </c>
-      <c r="Q26" s="3">
+      <c r="Q26" s="4">
         <v>42993</v>
       </c>
-      <c r="R26" s="3">
+      <c r="R26" s="4">
         <v>79152</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="T26" s="1" t="s">
-        <v>1</v>
+        <v>86</v>
       </c>
       <c r="U26" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V26" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G27" s="2">
         <v>8005353726</v>
@@ -2846,46 +2824,46 @@
       <c r="P27" s="1">
         <v>1200</v>
       </c>
-      <c r="Q27" s="3">
+      <c r="Q27" s="4">
         <v>44447</v>
       </c>
-      <c r="R27" s="3">
+      <c r="R27" s="4">
         <v>75857</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="T27" s="1" t="s">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="U27" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V27" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="H28" s="1">
         <v>100000</v>
@@ -2908,46 +2886,46 @@
       <c r="P28" s="1">
         <v>2304</v>
       </c>
-      <c r="Q28" s="3">
+      <c r="Q28" s="4">
         <v>41269</v>
       </c>
-      <c r="R28" s="3">
+      <c r="R28" s="4">
         <v>67932</v>
       </c>
       <c r="S28" s="1" t="s">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="T28" s="1" t="s">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="U28" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V28" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H29" s="1">
         <v>100000</v>
@@ -2970,46 +2948,46 @@
       <c r="P29" s="1">
         <v>3744</v>
       </c>
-      <c r="Q29" s="3">
+      <c r="Q29" s="4">
         <v>40704</v>
       </c>
-      <c r="R29" s="3">
+      <c r="R29" s="4">
         <v>68098</v>
       </c>
       <c r="S29" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="T29" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="U29" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="V29" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>220</v>
+        <v>95</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="H30" s="1">
         <v>300000</v>
@@ -3020,10 +2998,10 @@
       <c r="J30" s="1">
         <v>100000</v>
       </c>
-      <c r="K30" s="9">
+      <c r="K30" s="6">
         <v>200000</v>
       </c>
-      <c r="L30" s="9"/>
+      <c r="L30" s="6"/>
       <c r="M30" s="1" t="s">
         <v>1</v>
       </c>
@@ -3036,46 +3014,46 @@
       <c r="P30" s="1">
         <v>2400</v>
       </c>
-      <c r="Q30" s="3">
+      <c r="Q30" s="4">
         <v>41479</v>
       </c>
-      <c r="R30" s="3">
+      <c r="R30" s="4">
         <v>68142</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="T30" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="U30" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="V30" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H31" s="1">
         <v>55000</v>
@@ -3098,46 +3076,46 @@
       <c r="P31" s="1">
         <v>1200</v>
       </c>
-      <c r="Q31" s="3">
+      <c r="Q31" s="4">
         <v>40145</v>
       </c>
-      <c r="R31" s="3">
+      <c r="R31" s="4">
         <v>67173</v>
       </c>
       <c r="S31" s="1" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="U31" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="V31" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>221</v>
+        <v>101</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H32" s="1">
         <v>10000</v>
@@ -3160,43 +3138,43 @@
       <c r="P32" s="1">
         <v>1200</v>
       </c>
-      <c r="Q32" s="3">
+      <c r="Q32" s="4">
         <v>41535</v>
       </c>
-      <c r="R32" s="3">
+      <c r="R32" s="4">
         <v>67102</v>
       </c>
       <c r="S32" s="1" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="T32" s="1" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="U32" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="V32" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G33" s="2">
         <v>8009545212</v>
@@ -3222,46 +3200,46 @@
       <c r="P33" s="1">
         <v>3648</v>
       </c>
-      <c r="Q33" s="3">
+      <c r="Q33" s="4">
         <v>45779</v>
       </c>
-      <c r="R33" s="3">
+      <c r="R33" s="4">
         <v>56006</v>
       </c>
       <c r="S33" s="1" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="T33" s="1" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="U33" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="V33" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="V33" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.5">
-      <c r="A34" s="1" t="s">
-        <v>89</v>
-      </c>
       <c r="B34" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>222</v>
+        <v>104</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>97</v>
+        <v>58</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="H34" s="1">
         <v>200000</v>
@@ -3281,37 +3259,43 @@
       <c r="P34" s="1">
         <v>2520</v>
       </c>
-      <c r="Q34" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="R34" s="3" t="s">
-        <v>99</v>
+      <c r="Q34" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="R34" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="S34" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="T34" s="1" t="s">
+        <v>94</v>
       </c>
       <c r="U34" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.5">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>100</v>
+        <v>52</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>108</v>
       </c>
       <c r="H35" s="1">
         <v>100000</v>
@@ -3325,34 +3309,40 @@
       <c r="P35" s="1">
         <v>2760</v>
       </c>
-      <c r="Q35" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="R35" s="3" t="s">
-        <v>102</v>
+      <c r="Q35" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="R35" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="S35" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="T35" s="1" t="s">
+        <v>94</v>
       </c>
       <c r="U35" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.5">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G36" s="2">
         <v>8000474682</v>
@@ -3372,34 +3362,37 @@
       <c r="P36" s="1">
         <v>1800</v>
       </c>
-      <c r="Q36" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="R36" s="3" t="s">
-        <v>106</v>
+      <c r="Q36" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="R36" s="4" t="s">
+        <v>114</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.5">
+        <v>111</v>
+      </c>
+      <c r="T36" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G37" s="2">
         <v>8000474701</v>
@@ -3419,37 +3412,40 @@
       <c r="P37" s="1">
         <v>1800</v>
       </c>
-      <c r="Q37" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="R37" s="3" t="s">
-        <v>109</v>
+      <c r="Q37" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="R37" s="4" t="s">
+        <v>116</v>
       </c>
       <c r="S37" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
+      </c>
+      <c r="T37" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="U37" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.5">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G38" s="2">
         <v>8000474735</v>
@@ -3469,37 +3465,40 @@
       <c r="P38" s="1">
         <v>1800</v>
       </c>
-      <c r="Q38" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="R38" s="3" t="s">
+      <c r="Q38" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="R38" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="S38" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="S38" s="1" t="s">
-        <v>107</v>
+      <c r="T38" s="1" t="s">
+        <v>119</v>
       </c>
       <c r="U38" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39" spans="1:22" ht="63" x14ac:dyDescent="0.5">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="39" ht="63" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G39" s="2">
         <v>8000319947</v>
@@ -3522,34 +3521,40 @@
       <c r="P39" s="1">
         <v>7608</v>
       </c>
-      <c r="Q39" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="R39" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="U39" s="6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="Q39" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="R39" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="S39" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="T39" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="U39" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G40" s="2">
         <v>8001136733</v>
@@ -3572,34 +3577,37 @@
       <c r="P40" s="1">
         <v>2892</v>
       </c>
-      <c r="Q40" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="R40" s="3" t="s">
-        <v>118</v>
+      <c r="Q40" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="R40" s="4" t="s">
+        <v>126</v>
       </c>
       <c r="S40" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.5">
+        <v>124</v>
+      </c>
+      <c r="T40" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G41" s="2">
         <v>6000914783</v>
@@ -3616,34 +3624,40 @@
       <c r="P41" s="1">
         <v>2400</v>
       </c>
-      <c r="Q41" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="R41" s="3" t="s">
-        <v>121</v>
+      <c r="Q41" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="R41" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="S41" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="T41" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="U41" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.5">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G42" s="2">
         <v>8009554653</v>
@@ -3663,34 +3677,37 @@
       <c r="P42" s="1">
         <v>1764</v>
       </c>
-      <c r="Q42" s="3">
+      <c r="Q42" s="4">
         <v>45782</v>
       </c>
-      <c r="R42" s="3">
+      <c r="R42" s="4">
         <v>68427</v>
       </c>
       <c r="S42" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.5">
+        <v>124</v>
+      </c>
+      <c r="T42" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G43" s="2">
         <v>8006861955</v>
@@ -3707,37 +3724,43 @@
       <c r="P43" s="1">
         <v>2499.96</v>
       </c>
-      <c r="Q43" s="3">
+      <c r="Q43" s="4">
         <v>45200</v>
       </c>
-      <c r="R43" s="3">
+      <c r="R43" s="4">
         <v>61271</v>
       </c>
-      <c r="U43" s="6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="44" spans="1:22" ht="47.25" x14ac:dyDescent="0.5">
+      <c r="S43" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="T43" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="U43" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="44" ht="47.25" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G44" s="4" t="s">
-        <v>126</v>
+        <v>58</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>134</v>
       </c>
       <c r="H44" s="1">
         <v>100000</v>
@@ -3754,37 +3777,43 @@
       <c r="P44" s="1">
         <v>1800</v>
       </c>
-      <c r="Q44" s="7">
+      <c r="Q44" s="8">
         <v>40057</v>
       </c>
-      <c r="R44" s="3">
+      <c r="R44" s="4">
         <v>68181</v>
       </c>
-      <c r="U44" s="6" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="45" spans="1:22" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="S44" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="T44" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="U44" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="45" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>128</v>
+        <v>58</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>136</v>
       </c>
       <c r="H45" s="1">
         <v>160000</v>
@@ -3801,34 +3830,40 @@
       <c r="P45" s="1">
         <v>1200</v>
       </c>
-      <c r="Q45" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="R45" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="U45" s="6" t="s">
+      <c r="Q45" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="R45" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="S45" s="1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="T45" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="U45" s="3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G46" s="2">
         <v>8010004645</v>
@@ -3848,37 +3883,43 @@
       <c r="P46" s="1">
         <v>3000</v>
       </c>
-      <c r="Q46" s="3">
+      <c r="Q46" s="4">
         <v>45879</v>
       </c>
-      <c r="R46" s="3">
+      <c r="R46" s="4">
         <v>57202</v>
       </c>
+      <c r="S46" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="T46" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="U46" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.5">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G47" s="4" t="s">
-        <v>133</v>
+        <v>52</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>141</v>
       </c>
       <c r="H47" s="1">
         <v>1000000</v>
@@ -3892,37 +3933,43 @@
       <c r="P47" s="1">
         <v>5340</v>
       </c>
-      <c r="Q47" s="3">
+      <c r="Q47" s="4">
         <v>43378</v>
       </c>
-      <c r="R47" s="3">
+      <c r="R47" s="4">
         <v>68215</v>
       </c>
+      <c r="S47" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="T47" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="U47" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.5">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>136</v>
+        <v>58</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="H48" s="1">
         <v>100000</v>
@@ -3945,34 +3992,40 @@
       <c r="P48" s="1">
         <v>4368</v>
       </c>
-      <c r="Q48" s="3">
+      <c r="Q48" s="4">
         <v>40975</v>
       </c>
-      <c r="R48" s="3">
+      <c r="R48" s="4">
         <v>68368</v>
       </c>
+      <c r="S48" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="T48" s="1" t="s">
+        <v>143</v>
+      </c>
       <c r="U48" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="49" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="49" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G49" s="2">
         <v>6001549235</v>
@@ -3989,37 +4042,43 @@
       <c r="P49" s="1">
         <v>1440</v>
       </c>
-      <c r="Q49" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="R49" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="U49" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="50" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="Q49" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="R49" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="S49" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="T49" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="U49" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="50" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>142</v>
+        <v>58</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>150</v>
       </c>
       <c r="H50" s="1">
         <v>50000</v>
@@ -4033,37 +4092,43 @@
       <c r="P50" s="1">
         <v>1500</v>
       </c>
-      <c r="Q50" s="3" t="s">
+      <c r="Q50" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="R50" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="S50" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="R50" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="U50" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.5">
+      <c r="T50" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="U50" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G51" s="4" t="s">
-        <v>145</v>
+        <v>58</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>153</v>
       </c>
       <c r="H51" s="1">
         <v>150000</v>
@@ -4077,34 +4142,40 @@
       <c r="P51" s="1">
         <v>1200</v>
       </c>
-      <c r="Q51" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="R51" s="3" t="s">
-        <v>147</v>
+      <c r="Q51" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="R51" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="S51" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="T51" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="U51" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="52" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="52" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G52" s="2">
         <v>8005001007</v>
@@ -4121,34 +4192,40 @@
       <c r="P52" s="1">
         <v>2400</v>
       </c>
-      <c r="Q52" s="3">
+      <c r="Q52" s="4">
         <v>44413</v>
       </c>
-      <c r="R52" s="3">
+      <c r="R52" s="4">
         <v>61214</v>
       </c>
-      <c r="U52" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.5">
+      <c r="S52" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="T52" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="U52" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D53" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="G53" s="2">
         <v>8009518746</v>
@@ -4165,34 +4242,40 @@
       <c r="P53" s="1">
         <v>3132</v>
       </c>
-      <c r="Q53" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="R53" s="3" t="s">
-        <v>150</v>
+      <c r="Q53" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="R53" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="S53" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="T53" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="U53" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.5">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G54" s="2">
         <v>8005001052</v>
@@ -4209,34 +4292,40 @@
       <c r="P54" s="1">
         <v>6000</v>
       </c>
-      <c r="Q54" s="3">
+      <c r="Q54" s="4">
         <v>44201</v>
       </c>
-      <c r="R54" s="3">
+      <c r="R54" s="4">
         <v>56984</v>
       </c>
+      <c r="S54" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="T54" s="1" t="s">
+        <v>156</v>
+      </c>
       <c r="U54" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.5">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G55" s="2">
         <v>6001512162</v>
@@ -4253,34 +4342,40 @@
       <c r="P55" s="1">
         <v>1800</v>
       </c>
-      <c r="Q55" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="R55" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="U55" s="6" t="s">
+      <c r="Q55" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="R55" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="S55" s="1" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.5">
+      <c r="T55" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U55" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G56" s="2">
         <v>8002084775</v>
@@ -4297,37 +4392,43 @@
       <c r="P56" s="1">
         <v>12000</v>
       </c>
-      <c r="Q56" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="R56" s="3" t="s">
-        <v>159</v>
+      <c r="Q56" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="R56" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="S56" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="T56" s="1" t="s">
+        <v>165</v>
       </c>
       <c r="U56" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.5">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G57" s="4" t="s">
-        <v>161</v>
+        <v>52</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>169</v>
       </c>
       <c r="H57" s="1">
         <v>100000</v>
@@ -4335,45 +4436,51 @@
       <c r="I57" s="1">
         <v>100000</v>
       </c>
-      <c r="J57" s="9">
+      <c r="J57" s="6">
         <v>200000</v>
       </c>
-      <c r="K57" s="9"/>
-      <c r="L57" s="9"/>
+      <c r="K57" s="6"/>
+      <c r="L57" s="6"/>
       <c r="N57" s="1">
         <v>100000</v>
       </c>
       <c r="P57" s="1">
         <v>2400</v>
       </c>
-      <c r="Q57" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="R57" s="3" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="58" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="Q57" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="R57" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="S57" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="T57" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="58" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G58" s="4" t="s">
-        <v>164</v>
+        <v>58</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>172</v>
       </c>
       <c r="H58" s="1">
         <v>100000</v>
@@ -4387,37 +4494,43 @@
       <c r="P58" s="1">
         <v>1800</v>
       </c>
-      <c r="Q58" s="3">
+      <c r="Q58" s="4">
         <v>40158</v>
       </c>
-      <c r="R58" s="3">
+      <c r="R58" s="4">
         <v>68282</v>
       </c>
-      <c r="U58" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="59" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="S58" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="T58" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="U58" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="59" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G59" s="4" t="s">
-        <v>167</v>
+        <v>58</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>175</v>
       </c>
       <c r="H59" s="1">
         <v>150000</v>
@@ -4431,34 +4544,40 @@
       <c r="P59" s="1">
         <v>3000</v>
       </c>
-      <c r="Q59" s="3">
+      <c r="Q59" s="4">
         <v>41156</v>
       </c>
-      <c r="R59" s="3">
+      <c r="R59" s="4">
         <v>68184</v>
       </c>
-      <c r="U59" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.5">
+      <c r="S59" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="T59" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="U59" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G60" s="2">
         <v>8010660964</v>
@@ -4475,37 +4594,43 @@
       <c r="P60" s="1">
         <v>3672</v>
       </c>
-      <c r="Q60" s="3">
+      <c r="Q60" s="4">
         <v>46089</v>
       </c>
-      <c r="R60" s="3">
+      <c r="R60" s="4">
         <v>61064</v>
       </c>
+      <c r="S60" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="T60" s="1" t="s">
+        <v>168</v>
+      </c>
       <c r="U60" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.5">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G61" s="4" t="s">
-        <v>172</v>
+        <v>78</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>180</v>
       </c>
       <c r="H61" s="1">
         <v>500000</v>
@@ -4519,18 +4644,21 @@
       <c r="P61" s="1">
         <v>1800</v>
       </c>
-      <c r="Q61" s="3">
+      <c r="Q61" s="4">
         <v>44409</v>
       </c>
-      <c r="R61" s="3">
+      <c r="R61" s="4">
         <v>56097</v>
+      </c>
+      <c r="S61" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="T61" s="1" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="M1:V2 M3:O4 S3:V10 M33 B22:H22 S23:V25 A21:H21 B20:H20 T20:V22 S28:V33 B26:H27 T26:V27 S13:V19 M15:M17 B11:H12 T11:V12 A5 C5:H5 O5 O7 A6:H10 O9 O11 A13:H14 M5:M14 O14 A18:H19 O18 A23:H25 O23:O27 A28:H29 M18:M30 O30 J25 J19:J23 J12:J14 J10 J8 A15:H17 A33:H33 A1:J4 A30:C30 E30:H30 A31:H31 J31 M31 O31 A32:C32 J32 O32 E32:H32 J33 J15:J17 O15:O17" numberStoredAsText="1"/>
-  </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4538,164 +4666,161 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" customHeight="1"/>
   <cols>
     <col min="4" max="4" width="27.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B1" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="E1" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="F1" t="s">
         <v>1</v>
       </c>
       <c r="G1" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.5">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="D2" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="E2" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="G2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.5">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="B3" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D3" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="E3" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="G3" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.5">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B4" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="D4" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E4" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="G4" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.5">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B5" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="D5" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E5" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.5">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="B6" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="D6" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="E6" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.5">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="D7" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="E7" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.5">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="8" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="E8" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.5">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="9" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="E9" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:G2 A6:G7 A4:C4 E4:G4 A3:C3 E3:G3 A9:G9 A8:C8 E8:G8 A5:C5 E5:G5" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" customHeight="1"/>
   <cols>
     <col min="12" max="12" width="13.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>214</v>
       </c>
       <c r="B1" t="s">
         <v>4</v>
@@ -4719,42 +4844,42 @@
         <v>10</v>
       </c>
       <c r="I1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.5">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="B2" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="G2" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="H2">
         <v>500000</v>
@@ -4763,39 +4888,39 @@
         <v>6000</v>
       </c>
       <c r="J2" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="K2" t="s">
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="M2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.5">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="B3" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="C3" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="D3" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="G3" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="H3" t="s">
         <v>1</v>
@@ -4804,7 +4929,7 @@
         <v>3600</v>
       </c>
       <c r="J3" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="K3" t="s">
         <v>1</v>
@@ -4813,13 +4938,10 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:M3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ux: colourful benefit pills on each insurance policy row
Re-added benefit badges (Life Cover, CI, Medical, PA, TPD, etc.) with
keyword-based colours under each policy, for a more lively, scannable view.
</commit_message>
<xml_diff>
--- a/notion-import-templates/Insurance_Policies_Template.xlsx
+++ b/notion-import-templates/Insurance_Policies_Template.xlsx
@@ -1,17 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_BB2781936AF8E0F8718ED899919FF0B8BCB24D3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF8B9986-D34C-4542-A058-FE4083839E4D}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Insurance Policies" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Reference" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Sample" state="visible" r:id="rId6"/>
+    <sheet name="Insurance Policies" sheetId="1" r:id="rId1"/>
+    <sheet name="Reference" sheetId="2" r:id="rId2"/>
+    <sheet name="Sample" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -285,7 +287,7 @@
     <t>🛡️ Life Cover, ♿ TPD</t>
   </si>
   <si>
-    <t xml:space="preserve">1.LOH LI YAO
+    <t>1.LOH LI YAO
 2. CHAI YOKE FOONG</t>
   </si>
   <si>
@@ -388,7 +390,7 @@
     <t>22/09/2073</t>
   </si>
   <si>
-    <t xml:space="preserve">1. CHAN YUAN LIN
+    <t>1. CHAN YUAN LIN
 2. CHAN SHI LING
 3. CHAN CHEE KENG
 4. CHAN JIN HAO</t>
@@ -427,7 +429,7 @@
     <t>0102728587</t>
   </si>
   <si>
-    <t xml:space="preserve">1. LIM YEE FEI
+    <t>1. LIM YEE FEI
 2. LEONG AH LUAN
 3. LIM SHENG YEE</t>
   </si>
@@ -441,7 +443,7 @@
     <t>23/10/2086</t>
   </si>
   <si>
-    <t xml:space="preserve">1. LEONG AH LUAN
+    <t>1. LEONG AH LUAN
 2. LIM SHENG YEE</t>
   </si>
   <si>
@@ -472,7 +474,7 @@
     <t>15/07/2087</t>
   </si>
   <si>
-    <t xml:space="preserve">1. TOH HONG SHII
+    <t>1. TOH HONG SHII
 2. LIM BEE BEE</t>
   </si>
   <si>
@@ -545,7 +547,7 @@
     <t>0103101505</t>
   </si>
   <si>
-    <t xml:space="preserve">1. LEE YUK SONG
+    <t>1. LEE YUK SONG
 2. LIU KAI YOU</t>
   </si>
   <si>
@@ -711,24 +713,24 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -795,16 +797,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Table1" displayName="Table1" ref="P3:R33" totalsRowShown="1" headerRowCount="0">
-  <autoFilter ref="P3:R33">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="P3:R33" headerRowCount="0">
   <tableColumns count="3">
-    <tableColumn id="1" name="Annual Premium (MYR)"/>
-    <tableColumn id="2" name="Commencement Date"/>
-    <tableColumn id="3" name="Maturity Date"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Annual Premium (MYR)"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Commencement Date"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Maturity Date"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1131,33 +1128,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V61"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="27.25" style="1" customWidth="1"/>
+    <col min="1" max="1" width="27.265625" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="3" width="31.625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="31.59765625" style="1" customWidth="1"/>
     <col min="4" max="4" width="68" style="1" customWidth="1"/>
-    <col min="5" max="5" width="21.5" style="1" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="22.25" style="1" customWidth="1"/>
-    <col min="9" max="9" width="25.25" style="3" customWidth="1"/>
+    <col min="5" max="5" width="21.46484375" style="1" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="11.59765625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.59765625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="22.265625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="25.265625" style="3" customWidth="1"/>
     <col min="10" max="12" width="21" style="1" customWidth="1"/>
-    <col min="13" max="13" width="20.5" style="1" customWidth="1"/>
-    <col min="14" max="14" width="35.75" style="1" customWidth="1"/>
-    <col min="15" max="15" width="29.375" style="1" customWidth="1"/>
-    <col min="16" max="16" width="21.75" style="1" customWidth="1"/>
-    <col min="17" max="17" width="20.625" style="4" customWidth="1"/>
-    <col min="18" max="18" width="19.125" style="4" customWidth="1"/>
-    <col min="19" max="19" width="35.75" style="1" customWidth="1"/>
-    <col min="20" max="20" width="35.3125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="28.375" style="1" customWidth="1"/>
-    <col min="22" max="16384" width="9" style="1" customWidth="1"/>
+    <col min="13" max="13" width="20.46484375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="35.73046875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="29.3984375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="21.73046875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="20.59765625" style="4" customWidth="1"/>
+    <col min="18" max="18" width="19.1328125" style="4" customWidth="1"/>
+    <col min="19" max="19" width="35.73046875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="35.33203125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="28.3984375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="9" style="1" customWidth="1"/>
+    <col min="23" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1219,7 +1217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1281,7 +1279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1349,7 +1347,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
@@ -1417,7 +1415,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>47</v>
       </c>
@@ -1479,7 +1477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>47</v>
       </c>
@@ -1541,7 +1539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>47</v>
       </c>
@@ -1603,7 +1601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>62</v>
       </c>
@@ -1665,7 +1663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>66</v>
       </c>
@@ -1727,7 +1725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>66</v>
       </c>
@@ -1789,7 +1787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>71</v>
       </c>
@@ -1851,7 +1849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>71</v>
       </c>
@@ -1913,7 +1911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>71</v>
       </c>
@@ -1975,7 +1973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>71</v>
       </c>
@@ -2037,7 +2035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>71</v>
       </c>
@@ -2099,7 +2097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>71</v>
       </c>
@@ -2161,7 +2159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>74</v>
       </c>
@@ -2223,7 +2221,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>74</v>
       </c>
@@ -2285,7 +2283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>74</v>
       </c>
@@ -2347,7 +2345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>83</v>
       </c>
@@ -2409,7 +2407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>83</v>
       </c>
@@ -2471,7 +2469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>83</v>
       </c>
@@ -2533,7 +2531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>83</v>
       </c>
@@ -2595,7 +2593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>83</v>
       </c>
@@ -2657,7 +2655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>83</v>
       </c>
@@ -2719,7 +2717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>83</v>
       </c>
@@ -2781,7 +2779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>83</v>
       </c>
@@ -2843,7 +2841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>90</v>
       </c>
@@ -2905,7 +2903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>92</v>
       </c>
@@ -2967,7 +2965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>92</v>
       </c>
@@ -3033,7 +3031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>97</v>
       </c>
@@ -3095,7 +3093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>97</v>
       </c>
@@ -3157,7 +3155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
         <v>97</v>
       </c>
@@ -3219,7 +3217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
         <v>94</v>
       </c>
@@ -3275,7 +3273,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>94</v>
       </c>
@@ -3325,7 +3323,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
         <v>111</v>
       </c>
@@ -3375,7 +3373,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>111</v>
       </c>
@@ -3428,7 +3426,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A38" s="1" t="s">
         <v>111</v>
       </c>
@@ -3481,7 +3479,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="39" ht="63" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:22" ht="63" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
         <v>111</v>
       </c>
@@ -3537,7 +3535,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A40" s="1" t="s">
         <v>124</v>
       </c>
@@ -3590,7 +3588,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A41" s="1" t="s">
         <v>124</v>
       </c>
@@ -3640,7 +3638,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A42" s="1" t="s">
         <v>124</v>
       </c>
@@ -3690,7 +3688,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A43" s="1" t="s">
         <v>131</v>
       </c>
@@ -3740,7 +3738,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="44" ht="47.25" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:22" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="1" t="s">
         <v>131</v>
       </c>
@@ -3793,7 +3791,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="45" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:22" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="1" t="s">
         <v>131</v>
       </c>
@@ -3846,7 +3844,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A46" s="1" t="s">
         <v>131</v>
       </c>
@@ -3899,7 +3897,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A47" s="1" t="s">
         <v>140</v>
       </c>
@@ -3949,7 +3947,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A48" s="1" t="s">
         <v>143</v>
       </c>
@@ -4008,7 +4006,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="49" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="1" t="s">
         <v>143</v>
       </c>
@@ -4058,7 +4056,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="50" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="1" t="s">
         <v>143</v>
       </c>
@@ -4108,7 +4106,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A51" s="1" t="s">
         <v>143</v>
       </c>
@@ -4158,7 +4156,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="52" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="1" t="s">
         <v>143</v>
       </c>
@@ -4208,7 +4206,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A53" s="1" t="s">
         <v>156</v>
       </c>
@@ -4258,7 +4256,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A54" s="1" t="s">
         <v>156</v>
       </c>
@@ -4308,7 +4306,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A55" s="1" t="s">
         <v>156</v>
       </c>
@@ -4358,7 +4356,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A56" s="1" t="s">
         <v>165</v>
       </c>
@@ -4408,7 +4406,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A57" s="1" t="s">
         <v>168</v>
       </c>
@@ -4460,7 +4458,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="58" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="1" t="s">
         <v>168</v>
       </c>
@@ -4510,7 +4508,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="59" ht="31.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="1" t="s">
         <v>168</v>
       </c>
@@ -4560,7 +4558,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A60" s="1" t="s">
         <v>168</v>
       </c>
@@ -4610,7 +4608,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A61" s="1" t="s">
         <v>177</v>
       </c>
@@ -4666,14 +4664,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="4" max="4" width="27.25" customWidth="1"/>
+    <col min="4" max="4" width="27.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>181</v>
       </c>
@@ -4696,7 +4694,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>49</v>
       </c>
@@ -4713,7 +4711,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>189</v>
       </c>
@@ -4730,7 +4728,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>194</v>
       </c>
@@ -4747,7 +4745,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>199</v>
       </c>
@@ -4761,7 +4759,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>203</v>
       </c>
@@ -4775,7 +4773,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>81</v>
       </c>
@@ -4789,7 +4787,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="8" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="D8" t="s">
         <v>210</v>
       </c>
@@ -4797,7 +4795,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="9" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="D9" t="s">
         <v>212</v>
       </c>
@@ -4811,14 +4809,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="12" max="12" width="13.375" customWidth="1"/>
+    <col min="12" max="12" width="13.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>214</v>
       </c>
@@ -4859,7 +4857,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>215</v>
       </c>
@@ -4900,7 +4898,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>215</v>
       </c>

</xml_diff>

<commit_message>
Add Medical column to insurance listing + blank FA onboarding templates
- Insurance page: promote Medical Card (R&B / Annual Limit) from a sub-line
  to a dedicated column alongside Life/TPD, CI, Accident; align header,
  rows and subtotal across 8 columns
- Add FA_Onboarding_Templates/ — blank import templates (Clients, Insurance,
  Portfolio, CashFlow) with title/header/hint rows, all real client data
  cleared, for handing to other FAs in the Beta trial

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/Insurance_Policies_Template.xlsx
+++ b/notion-import-templates/Insurance_Policies_Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_BB2781936AF8E0F8718ED899919FF0B8BCB24D3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF8B9986-D34C-4542-A058-FE4083839E4D}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_BB2781936AF8E0F8718ED899919FF0B8BCB24D3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4D5306F-BFD6-448E-B21C-91B8A1C88C1A}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -733,12 +733,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -753,7 +759,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -778,6 +784,9 @@
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1148,7 +1157,7 @@
     <col min="16" max="16" width="21.73046875" style="1" customWidth="1"/>
     <col min="17" max="17" width="20.59765625" style="4" customWidth="1"/>
     <col min="18" max="18" width="19.1328125" style="4" customWidth="1"/>
-    <col min="19" max="19" width="35.73046875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="35.73046875" style="9" customWidth="1"/>
     <col min="20" max="20" width="35.33203125" style="1" customWidth="1"/>
     <col min="21" max="21" width="28.3984375" style="1" customWidth="1"/>
     <col min="22" max="22" width="9" style="1" customWidth="1"/>
@@ -1204,7 +1213,7 @@
       <c r="R1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="T1" s="1" t="s">
@@ -1266,7 +1275,7 @@
       <c r="R2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="S2" s="9" t="s">
         <v>1</v>
       </c>
       <c r="T2" s="1" t="s">
@@ -1334,7 +1343,7 @@
       <c r="R3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="1" t="s">
+      <c r="S3" s="9" t="s">
         <v>21</v>
       </c>
       <c r="T3" s="1" t="s">
@@ -1402,7 +1411,7 @@
       <c r="R4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="S4" s="1" t="s">
+      <c r="S4" s="9" t="s">
         <v>43</v>
       </c>
       <c r="T4" s="1" t="s">
@@ -1464,7 +1473,7 @@
       <c r="R5" s="4">
         <v>68281</v>
       </c>
-      <c r="S5" s="1" t="s">
+      <c r="S5" s="9" t="s">
         <v>54</v>
       </c>
       <c r="T5" s="1" t="s">
@@ -1526,7 +1535,7 @@
       <c r="R6" s="4">
         <v>68266</v>
       </c>
-      <c r="S6" s="1" t="s">
+      <c r="S6" s="9" t="s">
         <v>47</v>
       </c>
       <c r="T6" s="1" t="s">
@@ -1588,7 +1597,7 @@
       <c r="R7" s="4">
         <v>68319</v>
       </c>
-      <c r="S7" s="1" t="s">
+      <c r="S7" s="9" t="s">
         <v>47</v>
       </c>
       <c r="T7" s="1" t="s">
@@ -1650,7 +1659,7 @@
       <c r="R8" s="4">
         <v>60684</v>
       </c>
-      <c r="S8" s="1" t="s">
+      <c r="S8" s="9" t="s">
         <v>62</v>
       </c>
       <c r="T8" s="1" t="s">
@@ -1712,7 +1721,7 @@
       <c r="R9" s="4">
         <v>65263</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="S9" s="9" t="s">
         <v>66</v>
       </c>
       <c r="T9" s="1" t="s">
@@ -1774,7 +1783,7 @@
       <c r="R10" s="4">
         <v>54184</v>
       </c>
-      <c r="S10" s="1" t="s">
+      <c r="S10" s="9" t="s">
         <v>66</v>
       </c>
       <c r="T10" s="1" t="s">
@@ -1836,7 +1845,7 @@
       <c r="R11" s="4">
         <v>79103</v>
       </c>
-      <c r="S11" s="1" t="s">
+      <c r="S11" s="9" t="s">
         <v>71</v>
       </c>
       <c r="T11" s="1" t="s">
@@ -1898,7 +1907,7 @@
       <c r="R12" s="4">
         <v>71660</v>
       </c>
-      <c r="S12" s="1" t="s">
+      <c r="S12" s="9" t="s">
         <v>71</v>
       </c>
       <c r="T12" s="1" t="s">
@@ -1960,7 +1969,7 @@
       <c r="R13" s="4">
         <v>57415</v>
       </c>
-      <c r="S13" s="1" t="s">
+      <c r="S13" s="9" t="s">
         <v>71</v>
       </c>
       <c r="T13" s="1" t="s">
@@ -2022,7 +2031,7 @@
       <c r="R14" s="4">
         <v>64788</v>
       </c>
-      <c r="S14" s="1" t="s">
+      <c r="S14" s="9" t="s">
         <v>71</v>
       </c>
       <c r="T14" s="1" t="s">
@@ -2084,7 +2093,7 @@
       <c r="R15" s="4">
         <v>64529</v>
       </c>
-      <c r="S15" s="1" t="s">
+      <c r="S15" s="9" t="s">
         <v>71</v>
       </c>
       <c r="T15" s="1" t="s">
@@ -2146,7 +2155,7 @@
       <c r="R16" s="4">
         <v>57346</v>
       </c>
-      <c r="S16" s="1" t="s">
+      <c r="S16" s="9" t="s">
         <v>71</v>
       </c>
       <c r="T16" s="1" t="s">
@@ -2208,7 +2217,7 @@
       <c r="R17" s="4">
         <v>66355</v>
       </c>
-      <c r="S17" s="1" t="s">
+      <c r="S17" s="9" t="s">
         <v>74</v>
       </c>
       <c r="T17" s="1" t="s">
@@ -2270,7 +2279,7 @@
       <c r="R18" s="4">
         <v>66806</v>
       </c>
-      <c r="S18" s="1" t="s">
+      <c r="S18" s="9" t="s">
         <v>74</v>
       </c>
       <c r="T18" s="1" t="s">
@@ -2332,7 +2341,7 @@
       <c r="R19" s="4">
         <v>59241</v>
       </c>
-      <c r="S19" s="1" t="s">
+      <c r="S19" s="9" t="s">
         <v>74</v>
       </c>
       <c r="T19" s="1" t="s">
@@ -2394,7 +2403,7 @@
       <c r="R20" s="4">
         <v>69850</v>
       </c>
-      <c r="S20" s="1" t="s">
+      <c r="S20" s="9" t="s">
         <v>83</v>
       </c>
       <c r="T20" s="1" t="s">
@@ -2456,7 +2465,7 @@
       <c r="R21" s="4">
         <v>60719</v>
       </c>
-      <c r="S21" s="1" t="s">
+      <c r="S21" s="9" t="s">
         <v>83</v>
       </c>
       <c r="T21" s="1" t="s">
@@ -2518,7 +2527,7 @@
       <c r="R22" s="4">
         <v>68389</v>
       </c>
-      <c r="S22" s="1" t="s">
+      <c r="S22" s="9" t="s">
         <v>83</v>
       </c>
       <c r="T22" s="1" t="s">
@@ -2580,7 +2589,7 @@
       <c r="R23" s="4">
         <v>54816</v>
       </c>
-      <c r="S23" s="1" t="s">
+      <c r="S23" s="9" t="s">
         <v>83</v>
       </c>
       <c r="T23" s="1" t="s">
@@ -2642,7 +2651,7 @@
       <c r="R24" s="4">
         <v>68188</v>
       </c>
-      <c r="S24" s="1" t="s">
+      <c r="S24" s="9" t="s">
         <v>83</v>
       </c>
       <c r="T24" s="1" t="s">
@@ -2704,7 +2713,7 @@
       <c r="R25" s="4">
         <v>51423</v>
       </c>
-      <c r="S25" s="1" t="s">
+      <c r="S25" s="9" t="s">
         <v>83</v>
       </c>
       <c r="T25" s="1" t="s">
@@ -2766,7 +2775,7 @@
       <c r="R26" s="4">
         <v>79152</v>
       </c>
-      <c r="S26" s="1" t="s">
+      <c r="S26" s="9" t="s">
         <v>83</v>
       </c>
       <c r="T26" s="1" t="s">
@@ -2828,7 +2837,7 @@
       <c r="R27" s="4">
         <v>75857</v>
       </c>
-      <c r="S27" s="1" t="s">
+      <c r="S27" s="9" t="s">
         <v>83</v>
       </c>
       <c r="T27" s="1" t="s">
@@ -2890,7 +2899,7 @@
       <c r="R28" s="4">
         <v>67932</v>
       </c>
-      <c r="S28" s="1" t="s">
+      <c r="S28" s="9" t="s">
         <v>90</v>
       </c>
       <c r="T28" s="1" t="s">
@@ -2952,7 +2961,7 @@
       <c r="R29" s="4">
         <v>68098</v>
       </c>
-      <c r="S29" s="1" t="s">
+      <c r="S29" s="9" t="s">
         <v>92</v>
       </c>
       <c r="T29" s="1" t="s">
@@ -3018,7 +3027,7 @@
       <c r="R30" s="4">
         <v>68142</v>
       </c>
-      <c r="S30" s="1" t="s">
+      <c r="S30" s="9" t="s">
         <v>92</v>
       </c>
       <c r="T30" s="1" t="s">
@@ -3080,7 +3089,7 @@
       <c r="R31" s="4">
         <v>67173</v>
       </c>
-      <c r="S31" s="1" t="s">
+      <c r="S31" s="9" t="s">
         <v>97</v>
       </c>
       <c r="T31" s="1" t="s">
@@ -3142,7 +3151,7 @@
       <c r="R32" s="4">
         <v>67102</v>
       </c>
-      <c r="S32" s="1" t="s">
+      <c r="S32" s="9" t="s">
         <v>97</v>
       </c>
       <c r="T32" s="1" t="s">
@@ -3204,7 +3213,7 @@
       <c r="R33" s="4">
         <v>56006</v>
       </c>
-      <c r="S33" s="1" t="s">
+      <c r="S33" s="9" t="s">
         <v>97</v>
       </c>
       <c r="T33" s="1" t="s">
@@ -3263,7 +3272,7 @@
       <c r="R34" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="S34" s="1" t="s">
+      <c r="S34" s="9" t="s">
         <v>94</v>
       </c>
       <c r="T34" s="1" t="s">
@@ -3313,7 +3322,7 @@
       <c r="R35" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="S35" s="1" t="s">
+      <c r="S35" s="9" t="s">
         <v>94</v>
       </c>
       <c r="T35" s="1" t="s">
@@ -3366,7 +3375,7 @@
       <c r="R36" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="S36" s="1" t="s">
+      <c r="S36" s="9" t="s">
         <v>111</v>
       </c>
       <c r="T36" s="1" t="s">
@@ -3416,7 +3425,7 @@
       <c r="R37" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="S37" s="1" t="s">
+      <c r="S37" s="9" t="s">
         <v>111</v>
       </c>
       <c r="T37" s="1" t="s">
@@ -3469,7 +3478,7 @@
       <c r="R38" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="S38" s="1" t="s">
+      <c r="S38" s="9" t="s">
         <v>111</v>
       </c>
       <c r="T38" s="1" t="s">
@@ -3525,7 +3534,7 @@
       <c r="R39" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="S39" s="1" t="s">
+      <c r="S39" s="9" t="s">
         <v>111</v>
       </c>
       <c r="T39" s="1" t="s">
@@ -3581,7 +3590,7 @@
       <c r="R40" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="S40" s="1" t="s">
+      <c r="S40" s="9" t="s">
         <v>124</v>
       </c>
       <c r="T40" s="1" t="s">
@@ -3628,7 +3637,7 @@
       <c r="R41" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="S41" s="1" t="s">
+      <c r="S41" s="9" t="s">
         <v>124</v>
       </c>
       <c r="T41" s="1" t="s">
@@ -3681,7 +3690,7 @@
       <c r="R42" s="4">
         <v>68427</v>
       </c>
-      <c r="S42" s="1" t="s">
+      <c r="S42" s="9" t="s">
         <v>124</v>
       </c>
       <c r="T42" s="1" t="s">
@@ -3728,7 +3737,7 @@
       <c r="R43" s="4">
         <v>61271</v>
       </c>
-      <c r="S43" s="1" t="s">
+      <c r="S43" s="9" t="s">
         <v>131</v>
       </c>
       <c r="T43" s="1" t="s">
@@ -3781,7 +3790,7 @@
       <c r="R44" s="4">
         <v>68181</v>
       </c>
-      <c r="S44" s="1" t="s">
+      <c r="S44" s="9" t="s">
         <v>131</v>
       </c>
       <c r="T44" s="1" t="s">
@@ -3834,7 +3843,7 @@
       <c r="R45" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="S45" s="1" t="s">
+      <c r="S45" s="9" t="s">
         <v>131</v>
       </c>
       <c r="T45" s="1" t="s">
@@ -3887,7 +3896,7 @@
       <c r="R46" s="4">
         <v>57202</v>
       </c>
-      <c r="S46" s="1" t="s">
+      <c r="S46" s="9" t="s">
         <v>131</v>
       </c>
       <c r="T46" s="1" t="s">
@@ -3937,7 +3946,7 @@
       <c r="R47" s="4">
         <v>68215</v>
       </c>
-      <c r="S47" s="1" t="s">
+      <c r="S47" s="9" t="s">
         <v>140</v>
       </c>
       <c r="T47" s="1" t="s">
@@ -3996,7 +4005,7 @@
       <c r="R48" s="4">
         <v>68368</v>
       </c>
-      <c r="S48" s="1" t="s">
+      <c r="S48" s="9" t="s">
         <v>143</v>
       </c>
       <c r="T48" s="1" t="s">
@@ -4046,7 +4055,7 @@
       <c r="R49" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="S49" s="1" t="s">
+      <c r="S49" s="9" t="s">
         <v>143</v>
       </c>
       <c r="T49" s="1" t="s">
@@ -4096,7 +4105,7 @@
       <c r="R50" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="S50" s="1" t="s">
+      <c r="S50" s="9" t="s">
         <v>143</v>
       </c>
       <c r="T50" s="1" t="s">
@@ -4146,7 +4155,7 @@
       <c r="R51" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="S51" s="1" t="s">
+      <c r="S51" s="9" t="s">
         <v>143</v>
       </c>
       <c r="T51" s="1" t="s">
@@ -4196,7 +4205,7 @@
       <c r="R52" s="4">
         <v>61214</v>
       </c>
-      <c r="S52" s="1" t="s">
+      <c r="S52" s="9" t="s">
         <v>143</v>
       </c>
       <c r="T52" s="1" t="s">
@@ -4246,7 +4255,7 @@
       <c r="R53" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="S53" s="1" t="s">
+      <c r="S53" s="9" t="s">
         <v>156</v>
       </c>
       <c r="T53" s="1" t="s">
@@ -4296,7 +4305,7 @@
       <c r="R54" s="4">
         <v>56984</v>
       </c>
-      <c r="S54" s="1" t="s">
+      <c r="S54" s="9" t="s">
         <v>156</v>
       </c>
       <c r="T54" s="1" t="s">
@@ -4346,7 +4355,7 @@
       <c r="R55" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="S55" s="1" t="s">
+      <c r="S55" s="9" t="s">
         <v>156</v>
       </c>
       <c r="T55" s="1" t="s">
@@ -4396,7 +4405,7 @@
       <c r="R56" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="S56" s="1" t="s">
+      <c r="S56" s="9" t="s">
         <v>165</v>
       </c>
       <c r="T56" s="1" t="s">
@@ -4451,7 +4460,7 @@
       <c r="R57" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="S57" s="1" t="s">
+      <c r="S57" s="9" t="s">
         <v>168</v>
       </c>
       <c r="T57" s="1" t="s">
@@ -4498,7 +4507,7 @@
       <c r="R58" s="4">
         <v>68282</v>
       </c>
-      <c r="S58" s="1" t="s">
+      <c r="S58" s="9" t="s">
         <v>168</v>
       </c>
       <c r="T58" s="1" t="s">
@@ -4548,7 +4557,7 @@
       <c r="R59" s="4">
         <v>68184</v>
       </c>
-      <c r="S59" s="1" t="s">
+      <c r="S59" s="9" t="s">
         <v>168</v>
       </c>
       <c r="T59" s="1" t="s">
@@ -4598,7 +4607,7 @@
       <c r="R60" s="4">
         <v>61064</v>
       </c>
-      <c r="S60" s="1" t="s">
+      <c r="S60" s="9" t="s">
         <v>168</v>
       </c>
       <c r="T60" s="1" t="s">
@@ -4648,7 +4657,7 @@
       <c r="R61" s="4">
         <v>56097</v>
       </c>
-      <c r="S61" s="1" t="s">
+      <c r="S61" s="9" t="s">
         <v>177</v>
       </c>
       <c r="T61" s="1" t="s">

</xml_diff>